<commit_message>
Weekly economic data update
</commit_message>
<xml_diff>
--- a/Economic_Metrics_All_Metros.xlsx
+++ b/Economic_Metrics_All_Metros.xlsx
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>70.2</v>
+        <v>70.3</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>68.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>64.40000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>62.7</v>
+        <v>62.6</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>60.9</v>
+        <v>61.8</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>57.4</v>
+        <v>57.5</v>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F13" s="8" t="n">
-        <v>57.1</v>
+        <v>57</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="F14" s="8" t="n">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="F16" s="8" t="n">
-        <v>54.7</v>
+        <v>54.8</v>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
@@ -1105,16 +1105,16 @@
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Philadelphia-Camden-Wilmington</t>
+          <t>Seattle-Tacoma-Bellevue</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>52.6</v>
+        <v>52.9</v>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
@@ -1136,16 +1136,16 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Seattle-Tacoma-Bellevue</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="F18" s="8" t="n">
-        <v>52.9</v>
+        <v>53.2</v>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
@@ -1167,16 +1167,16 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="F19" s="8" t="n">
-        <v>53.2</v>
+        <v>52.6</v>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
@@ -1198,20 +1198,20 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Philadelphia-Camden-Wilmington</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="F20" s="8" t="n">
-        <v>52.7</v>
+        <v>52.5</v>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="F22" s="8" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="F27" s="11" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="F28" s="11" t="n">
-        <v>46.8</v>
+        <v>46.6</v>
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="F29" s="11" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="F31" s="11" t="n">
-        <v>46.1</v>
+        <v>45.9</v>
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="F32" s="11" t="n">
-        <v>45.1</v>
+        <v>45.2</v>
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="F33" s="11" t="n">
-        <v>43.7</v>
+        <v>43.6</v>
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="F34" s="11" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="F35" s="11" t="n">
-        <v>42.3</v>
+        <v>42.4</v>
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="F37" s="11" t="n">
-        <v>40.7</v>
+        <v>40.6</v>
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="F40" s="14" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="G40" s="15" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="F41" s="14" t="n">
-        <v>36.1</v>
+        <v>36</v>
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="F44" s="14" t="n">
-        <v>35.3</v>
+        <v>35.1</v>
       </c>
       <c r="G44" s="15" t="inlineStr">
         <is>
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="F45" s="14" t="n">
-        <v>35.3</v>
+        <v>35.2</v>
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="F46" s="14" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="G46" s="15" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="F47" s="14" t="n">
-        <v>33.9</v>
+        <v>33.8</v>
       </c>
       <c r="G47" s="15" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="F48" s="14" t="n">
-        <v>32.3</v>
+        <v>32.2</v>
       </c>
       <c r="G48" s="15" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="F49" s="14" t="n">
-        <v>30.7</v>
+        <v>30.6</v>
       </c>
       <c r="G49" s="15" t="inlineStr">
         <is>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="F51" s="17" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="G51" s="18" t="inlineStr">
         <is>
@@ -2341,7 +2341,7 @@
         <v>80</v>
       </c>
       <c r="D3" s="22" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E3" s="21" t="n">
         <v>74</v>
@@ -2380,8 +2380,8 @@
       <c r="C4" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="23" t="n">
-        <v>69</v>
+      <c r="D4" s="21" t="n">
+        <v>70</v>
       </c>
       <c r="E4" s="23" t="n">
         <v>62</v>
@@ -2501,7 +2501,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>46</v>
@@ -2541,7 +2541,7 @@
         <v>86</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" s="23" t="n">
         <v>56</v>
@@ -2581,7 +2581,7 @@
         <v>86</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>52</v>
@@ -2615,13 +2615,13 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="21" t="n">
         <v>80</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>94</v>
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>68</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" s="22" t="n">
         <v>18</v>
@@ -2741,7 +2741,7 @@
         <v>50</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="22" t="n">
         <v>28</v>
@@ -2781,7 +2781,7 @@
         <v>94</v>
       </c>
       <c r="D14" s="23" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" s="22" t="n">
         <v>6</v>
@@ -2891,161 +2891,161 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Philadelphia-Camden-Wilmington</t>
+          <t>Seattle-Tacoma-Bellevue</t>
         </is>
       </c>
       <c r="B17" s="20" t="n">
         <v>53</v>
       </c>
       <c r="C17" s="22" t="n">
-        <v>34</v>
-      </c>
-      <c r="D17" s="22" t="n">
-        <v>43</v>
-      </c>
-      <c r="E17" s="22" t="n">
-        <v>34</v>
+        <v>6</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>84</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>92</v>
       </c>
       <c r="F17" s="22" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G17" s="21" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H17" s="21" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I17" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="J17" s="21" t="n">
-        <v>70</v>
-      </c>
-      <c r="K17" s="21" t="n">
-        <v>70</v>
-      </c>
-      <c r="L17" s="23" t="n">
         <v>64</v>
+      </c>
+      <c r="J17" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="K17" s="23" t="n">
+        <v>66</v>
+      </c>
+      <c r="L17" s="22" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Seattle-Tacoma-Bellevue</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="B18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="C18" s="22" t="n">
-        <v>6</v>
-      </c>
-      <c r="D18" s="21" t="n">
-        <v>84</v>
+      <c r="C18" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="22" t="n">
+        <v>10</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>92</v>
-      </c>
-      <c r="F18" s="22" t="n">
-        <v>30</v>
+        <v>96</v>
+      </c>
+      <c r="F18" s="21" t="n">
+        <v>76</v>
       </c>
       <c r="G18" s="21" t="n">
-        <v>78</v>
-      </c>
-      <c r="H18" s="21" t="n">
+        <v>80</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="I18" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="J18" s="21" t="n">
         <v>76</v>
       </c>
-      <c r="I18" s="23" t="n">
-        <v>64</v>
-      </c>
-      <c r="J18" s="22" t="n">
-        <v>16</v>
-      </c>
-      <c r="K18" s="23" t="n">
-        <v>66</v>
+      <c r="K18" s="21" t="n">
+        <v>86</v>
       </c>
       <c r="L18" s="22" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="B19" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="C19" s="23" t="n">
-        <v>50</v>
+      <c r="C19" s="21" t="n">
+        <v>98</v>
       </c>
       <c r="D19" s="22" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" s="21" t="n">
-        <v>96</v>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>76</v>
-      </c>
-      <c r="G19" s="21" t="n">
-        <v>80</v>
-      </c>
-      <c r="H19" s="22" t="n">
-        <v>44</v>
-      </c>
-      <c r="I19" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="J19" s="21" t="n">
-        <v>76</v>
-      </c>
-      <c r="K19" s="21" t="n">
-        <v>86</v>
+      <c r="E19" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="21" t="n">
+        <v>92</v>
+      </c>
+      <c r="I19" s="21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" s="23" t="n">
+        <v>68</v>
+      </c>
+      <c r="K19" s="23" t="n">
+        <v>60</v>
       </c>
       <c r="L19" s="22" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Philadelphia-Camden-Wilmington</t>
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>53</v>
-      </c>
-      <c r="C20" s="21" t="n">
-        <v>98</v>
+        <v>52</v>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>34</v>
       </c>
       <c r="D20" s="22" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E20" s="22" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="F20" s="22" t="n">
-        <v>12</v>
-      </c>
-      <c r="G20" s="22" t="n">
-        <v>20</v>
+        <v>32</v>
+      </c>
+      <c r="G20" s="21" t="n">
+        <v>86</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>92</v>
-      </c>
-      <c r="I20" s="21" t="n">
-        <v>90</v>
-      </c>
-      <c r="J20" s="23" t="n">
-        <v>68</v>
-      </c>
-      <c r="K20" s="23" t="n">
-        <v>60</v>
-      </c>
-      <c r="L20" s="22" t="n">
-        <v>18</v>
+        <v>80</v>
+      </c>
+      <c r="I20" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="J20" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="K20" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="L20" s="23" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="21">
@@ -3101,7 +3101,7 @@
         <v>50</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E22" s="22" t="n">
         <v>20</v>
@@ -3301,7 +3301,7 @@
         <v>50</v>
       </c>
       <c r="D27" s="22" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E27" s="22" t="n">
         <v>22</v>
@@ -3341,7 +3341,7 @@
         <v>30</v>
       </c>
       <c r="D28" s="23" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E28" s="22" t="n">
         <v>40</v>
@@ -3381,7 +3381,7 @@
         <v>68</v>
       </c>
       <c r="D29" s="21" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E29" s="23" t="n">
         <v>60</v>
@@ -3461,7 +3461,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="23" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E31" s="22" t="n">
         <v>16</v>
@@ -3501,7 +3501,7 @@
         <v>2</v>
       </c>
       <c r="D32" s="23" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E32" s="21" t="n">
         <v>82</v>
@@ -3541,7 +3541,7 @@
         <v>68</v>
       </c>
       <c r="D33" s="22" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E33" s="21" t="n">
         <v>86</v>
@@ -3621,7 +3621,7 @@
         <v>20</v>
       </c>
       <c r="D35" s="23" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E35" s="22" t="n">
         <v>42</v>
@@ -3821,7 +3821,7 @@
         <v>50</v>
       </c>
       <c r="D40" s="23" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E40" s="22" t="n">
         <v>2</v>
@@ -3861,7 +3861,7 @@
         <v>24</v>
       </c>
       <c r="D41" s="22" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E41" s="22" t="n">
         <v>12</v>
@@ -3981,7 +3981,7 @@
         <v>32</v>
       </c>
       <c r="D44" s="23" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E44" s="22" t="n">
         <v>14</v>
@@ -4021,7 +4021,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="22" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E45" s="22" t="n">
         <v>32</v>
@@ -4061,7 +4061,7 @@
         <v>8</v>
       </c>
       <c r="D46" s="21" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E46" s="23" t="n">
         <v>64</v>
@@ -4141,7 +4141,7 @@
         <v>20</v>
       </c>
       <c r="D48" s="22" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E48" s="23" t="n">
         <v>66</v>
@@ -4181,7 +4181,7 @@
         <v>10</v>
       </c>
       <c r="D49" s="22" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E49" s="21" t="n">
         <v>76</v>
@@ -4722,13 +4722,15 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>61 (B+)</t>
+          <t>62 (B+)</t>
         </is>
       </c>
       <c r="C10" s="24" t="n">
         <v>3.3</v>
       </c>
-      <c r="D10" s="24" t="n"/>
+      <c r="D10" s="24" t="n">
+        <v>64.56999999999999</v>
+      </c>
       <c r="E10" s="24" t="n">
         <v>8.27</v>
       </c>
@@ -4804,7 +4806,7 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>57 (B)</t>
+          <t>58 (B)</t>
         </is>
       </c>
       <c r="C12" s="24" t="n">
@@ -5009,7 +5011,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Philadelphia-Camden-Wilmington</t>
+          <t>Seattle-Tacoma-Bellevue</t>
         </is>
       </c>
       <c r="B17" s="25" t="inlineStr">
@@ -5018,40 +5020,40 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17" s="24" t="n">
-        <v>63.96</v>
+        <v>68.23999999999999</v>
       </c>
       <c r="E17" s="24" t="n">
-        <v>2.21</v>
+        <v>7.63</v>
       </c>
       <c r="F17" s="24" t="n">
-        <v>5.41</v>
+        <v>5.53</v>
       </c>
       <c r="G17" s="24" t="n">
-        <v>3.56</v>
+        <v>3.26</v>
       </c>
       <c r="H17" s="24" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="I17" s="24" t="n">
-        <v>1.56</v>
+        <v>9.73</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>14.25</v>
+        <v>-0.14</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.44</v>
+        <v>0.23</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Seattle-Tacoma-Bellevue</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="B18" s="25" t="inlineStr">
@@ -5060,40 +5062,40 @@
         </is>
       </c>
       <c r="C18" s="24" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="D18" s="24" t="n">
-        <v>68.23999999999999</v>
+        <v>60.33</v>
       </c>
       <c r="E18" s="24" t="n">
-        <v>7.63</v>
+        <v>8.65</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>5.53</v>
+        <v>4.17</v>
       </c>
       <c r="G18" s="24" t="n">
-        <v>3.26</v>
+        <v>3.38</v>
       </c>
       <c r="H18" s="24" t="n">
-        <v>34.8</v>
+        <v>33.9</v>
       </c>
       <c r="I18" s="24" t="n">
-        <v>9.73</v>
+        <v>-18.72</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>-0.14</v>
+        <v>15.05</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.23</v>
+        <v>3.76</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="B19" s="25" t="inlineStr">
@@ -5102,76 +5104,76 @@
         </is>
       </c>
       <c r="C19" s="24" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="D19" s="24" t="n">
-        <v>60.33</v>
+        <v>60.56</v>
       </c>
       <c r="E19" s="24" t="n">
-        <v>8.65</v>
+        <v>-0.12</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>4.17</v>
+        <v>7.12</v>
       </c>
       <c r="G19" s="24" t="n">
-        <v>3.38</v>
+        <v>1.44</v>
       </c>
       <c r="H19" s="24" t="n">
-        <v>33.9</v>
+        <v>35.5</v>
       </c>
       <c r="I19" s="24" t="n">
-        <v>-18.72</v>
+        <v>32.24</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>15.05</v>
+        <v>10.88</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>3.76</v>
+        <v>-0.21</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Philadelphia-Camden-Wilmington</t>
         </is>
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>53 (B)</t>
+          <t>52 (B)</t>
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="D20" s="24" t="n">
-        <v>60.56</v>
+        <v>63.96</v>
       </c>
       <c r="E20" s="24" t="n">
-        <v>-0.12</v>
+        <v>2.21</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>7.12</v>
+        <v>5.41</v>
       </c>
       <c r="G20" s="24" t="n">
-        <v>1.44</v>
+        <v>3.56</v>
       </c>
       <c r="H20" s="24" t="n">
-        <v>35.5</v>
+        <v>34.9</v>
       </c>
       <c r="I20" s="24" t="n">
-        <v>32.24</v>
+        <v>1.56</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>10.88</v>
+        <v>14.25</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>-0.21</v>
+        <v>0.44</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21">
@@ -6575,7 +6577,7 @@
         </is>
       </c>
       <c r="F2" s="14" t="n">
-        <v>32.3</v>
+        <v>32.2</v>
       </c>
       <c r="G2" s="14" t="n">
         <v>4.5</v>
@@ -6613,7 +6615,7 @@
         </is>
       </c>
       <c r="F3" s="14" t="n">
-        <v>30.7</v>
+        <v>30.6</v>
       </c>
       <c r="G3" s="14" t="n">
         <v>4.8</v>
@@ -6651,7 +6653,7 @@
         </is>
       </c>
       <c r="F4" s="11" t="n">
-        <v>42.3</v>
+        <v>42.4</v>
       </c>
       <c r="G4" s="11" t="n">
         <v>4.5</v>
@@ -6727,7 +6729,7 @@
         </is>
       </c>
       <c r="F6" s="11" t="n">
-        <v>46.8</v>
+        <v>46.6</v>
       </c>
       <c r="G6" s="11" t="n">
         <v>4.2</v>
@@ -6765,7 +6767,7 @@
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>43.7</v>
+        <v>43.6</v>
       </c>
       <c r="G7" s="11" t="n">
         <v>3.5</v>
@@ -6803,7 +6805,7 @@
         </is>
       </c>
       <c r="F8" s="11" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G8" s="11" t="n">
         <v>3.8</v>
@@ -6833,7 +6835,7 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
@@ -6841,12 +6843,14 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>60.9</v>
+        <v>61.8</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>3.3</v>
       </c>
-      <c r="H9" s="5" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>64.56999999999999</v>
+      </c>
       <c r="I9" s="5" t="n">
         <v>8.27</v>
       </c>
@@ -6869,7 +6873,7 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
@@ -6877,7 +6881,7 @@
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>4</v>
@@ -6915,7 +6919,7 @@
         </is>
       </c>
       <c r="F11" s="11" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="G11" s="11" t="n">
         <v>3.5</v>
@@ -7029,7 +7033,7 @@
         </is>
       </c>
       <c r="F14" s="14" t="n">
-        <v>35.3</v>
+        <v>35.1</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>4.1</v>
@@ -7067,7 +7071,7 @@
         </is>
       </c>
       <c r="F15" s="11" t="n">
-        <v>40.7</v>
+        <v>40.6</v>
       </c>
       <c r="G15" s="11" t="n">
         <v>4.7</v>
@@ -7219,7 +7223,7 @@
         </is>
       </c>
       <c r="F19" s="17" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="G19" s="17" t="n">
         <v>4.4</v>
@@ -7295,7 +7299,7 @@
         </is>
       </c>
       <c r="F21" s="14" t="n">
-        <v>36.1</v>
+        <v>36</v>
       </c>
       <c r="G21" s="14" t="n">
         <v>4.4</v>
@@ -7333,7 +7337,7 @@
         </is>
       </c>
       <c r="F22" s="14" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>3.6</v>
@@ -7371,7 +7375,7 @@
         </is>
       </c>
       <c r="F23" s="11" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="G23" s="11" t="n">
         <v>3.6</v>
@@ -7401,7 +7405,7 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
@@ -7409,7 +7413,7 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>57.4</v>
+        <v>57.5</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>3.5</v>
@@ -7447,7 +7451,7 @@
         </is>
       </c>
       <c r="F25" s="14" t="n">
-        <v>35.3</v>
+        <v>35.2</v>
       </c>
       <c r="G25" s="14" t="n">
         <v>3.7</v>
@@ -7523,7 +7527,7 @@
         </is>
       </c>
       <c r="F27" s="14" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>4.9</v>
@@ -7637,7 +7641,7 @@
         </is>
       </c>
       <c r="F30" s="11" t="n">
-        <v>45.1</v>
+        <v>45.2</v>
       </c>
       <c r="G30" s="11" t="n">
         <v>5.2</v>
@@ -7675,7 +7679,7 @@
         </is>
       </c>
       <c r="F31" s="8" t="n">
-        <v>57.1</v>
+        <v>57</v>
       </c>
       <c r="G31" s="8" t="n">
         <v>3.6</v>
@@ -7713,7 +7717,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>3.5</v>
@@ -7751,7 +7755,7 @@
         </is>
       </c>
       <c r="F33" s="8" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>3.6</v>
@@ -7789,7 +7793,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>70.2</v>
+        <v>70.3</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>2.5</v>
@@ -7901,7 +7905,7 @@
         </is>
       </c>
       <c r="F37" s="11" t="n">
-        <v>46.1</v>
+        <v>45.9</v>
       </c>
       <c r="G37" s="11" t="n">
         <v>4</v>
@@ -8053,7 +8057,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="G41" s="5" t="n">
         <v>3.1</v>
@@ -8091,7 +8095,7 @@
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>54.7</v>
+        <v>54.8</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>3</v>
@@ -8129,7 +8133,7 @@
         </is>
       </c>
       <c r="F43" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="G43" s="5" t="n">
         <v>3.6</v>
@@ -8167,7 +8171,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>62.7</v>
+        <v>62.6</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>3.1</v>
@@ -8205,7 +8209,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>68.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>3.3</v>
@@ -8243,7 +8247,7 @@
         </is>
       </c>
       <c r="F46" s="14" t="n">
-        <v>33.9</v>
+        <v>33.8</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>4</v>
@@ -8319,7 +8323,7 @@
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="G48" s="8" t="n">
         <v>2.2</v>
@@ -8395,7 +8399,7 @@
         </is>
       </c>
       <c r="F50" s="5" t="n">
-        <v>64.40000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>4</v>
@@ -8433,7 +8437,7 @@
         </is>
       </c>
       <c r="F51" s="8" t="n">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="G51" s="8" t="n">
         <v>2.7</v>
@@ -8808,7 +8812,7 @@
         </is>
       </c>
       <c r="C11" s="30" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: Align READMEs and scoring engine metadata with actual codebase
- Update `README.md` to reference the correct pipeline script `city_econ_pipeline.py`.
- Update `SCORING_README.md` to detail the Unemployment Rate Composite (101A) and Civilian Labor Force YoY Growth (102A) design, replacing the outdated LFP descriptions and aligning the metric weights/category summaries.
- Update `calculate_metrics_reconciled_V6.py` and output JSON with corrected metadata notes, weights, version, and spreadsheet headers.
- Remove deprecated 106D metric from Excel Sheet 2 column config to avoid blank column drift.

Co-authored-by: danielwipert <13682174+danielwipert@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Economic_Metrics_All_Metros.xlsx
+++ b/Economic_Metrics_All_Metros.xlsx
@@ -228,10 +228,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2226,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2239,7 +2239,6 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2262,7 +2261,7 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>102A
-(LFP)</t>
+(CLF YoY)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2285,26 +2284,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>106D
-(Weekly Hours)</t>
+          <t>107E
+(Labor Demand)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>107E
-(Emp Growth YoY)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>200B
 (Permits YoY)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>204A
-(DoM YoY)</t>
+(DoM)</t>
         </is>
       </c>
     </row>
@@ -2332,14 +2325,13 @@
       <c r="G2" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="H2" s="32" t="n"/>
+      <c r="H2" s="30" t="n">
+        <v>98</v>
+      </c>
       <c r="I2" s="30" t="n">
-        <v>98</v>
-      </c>
-      <c r="J2" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="K2" s="33" t="n">
+      <c r="J2" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2364,17 +2356,16 @@
       <c r="F3" s="30" t="n">
         <v>71</v>
       </c>
-      <c r="G3" s="33" t="n">
+      <c r="G3" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="H3" s="32" t="n"/>
+      <c r="H3" s="30" t="n">
+        <v>84</v>
+      </c>
       <c r="I3" s="30" t="n">
-        <v>84</v>
-      </c>
-      <c r="J3" s="30" t="n">
         <v>78</v>
       </c>
-      <c r="K3" s="33" t="n">
+      <c r="J3" s="32" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2402,14 +2393,13 @@
       <c r="G4" s="30" t="n">
         <v>78</v>
       </c>
-      <c r="H4" s="32" t="n"/>
-      <c r="I4" s="30" t="n">
+      <c r="H4" s="30" t="n">
         <v>92</v>
       </c>
-      <c r="J4" s="33" t="n">
+      <c r="I4" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="31" t="n">
+      <c r="J4" s="31" t="n">
         <v>66</v>
       </c>
     </row>
@@ -2425,7 +2415,7 @@
       <c r="C5" s="30" t="n">
         <v>92</v>
       </c>
-      <c r="D5" s="33" t="n">
+      <c r="D5" s="32" t="n">
         <v>49</v>
       </c>
       <c r="E5" s="30" t="n">
@@ -2434,17 +2424,16 @@
       <c r="F5" s="30" t="n">
         <v>92</v>
       </c>
-      <c r="G5" s="33" t="n">
+      <c r="G5" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="H5" s="32" t="n"/>
-      <c r="I5" s="33" t="n">
+      <c r="H5" s="32" t="n">
         <v>48</v>
       </c>
+      <c r="I5" s="30" t="n">
+        <v>88</v>
+      </c>
       <c r="J5" s="30" t="n">
-        <v>88</v>
-      </c>
-      <c r="K5" s="30" t="n">
         <v>96</v>
       </c>
     </row>
@@ -2469,17 +2458,16 @@
       <c r="F6" s="30" t="n">
         <v>90</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G6" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="H6" s="32" t="n"/>
-      <c r="I6" s="30" t="n">
+      <c r="H6" s="30" t="n">
         <v>72</v>
       </c>
-      <c r="J6" s="31" t="n">
+      <c r="I6" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="K6" s="33" t="n">
+      <c r="J6" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2495,7 +2483,7 @@
       <c r="C7" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="D7" s="33" t="n">
+      <c r="D7" s="32" t="n">
         <v>41</v>
       </c>
       <c r="E7" s="30" t="n">
@@ -2507,14 +2495,13 @@
       <c r="G7" s="30" t="n">
         <v>88</v>
       </c>
-      <c r="H7" s="32" t="n"/>
-      <c r="I7" s="30" t="n">
+      <c r="H7" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="J7" s="33" t="n">
+      <c r="I7" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="33" t="n">
+      <c r="J7" s="32" t="n">
         <v>48</v>
       </c>
     </row>
@@ -2542,14 +2529,13 @@
       <c r="G8" s="30" t="n">
         <v>96</v>
       </c>
-      <c r="H8" s="32" t="n"/>
-      <c r="I8" s="30" t="n">
+      <c r="H8" s="30" t="n">
         <v>90</v>
       </c>
-      <c r="J8" s="33" t="n">
+      <c r="I8" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="K8" s="31" t="n">
+      <c r="J8" s="31" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2568,23 +2554,22 @@
       <c r="D9" s="31" t="n">
         <v>65</v>
       </c>
-      <c r="E9" s="33" t="n">
+      <c r="E9" s="32" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="30" t="n">
         <v>76</v>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="H9" s="32" t="n"/>
-      <c r="I9" s="31" t="n">
+      <c r="H9" s="31" t="n">
         <v>62</v>
       </c>
+      <c r="I9" s="30" t="n">
+        <v>76</v>
+      </c>
       <c r="J9" s="30" t="n">
-        <v>76</v>
-      </c>
-      <c r="K9" s="30" t="n">
         <v>94</v>
       </c>
     </row>
@@ -2603,23 +2588,22 @@
       <c r="D10" s="30" t="n">
         <v>88</v>
       </c>
-      <c r="E10" s="33" t="n">
+      <c r="E10" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="F10" s="33" t="n">
+      <c r="F10" s="32" t="n">
         <v>47</v>
       </c>
       <c r="G10" s="31" t="n">
         <v>64</v>
       </c>
-      <c r="H10" s="32" t="n"/>
+      <c r="H10" s="30" t="n">
+        <v>70</v>
+      </c>
       <c r="I10" s="30" t="n">
-        <v>70</v>
-      </c>
-      <c r="J10" s="30" t="n">
         <v>72</v>
       </c>
-      <c r="K10" s="31" t="n">
+      <c r="J10" s="31" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2632,7 +2616,7 @@
       <c r="B11" s="29" t="n">
         <v>62</v>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="32" t="n">
         <v>36</v>
       </c>
       <c r="D11" s="30" t="n">
@@ -2647,14 +2631,13 @@
       <c r="G11" s="30" t="n">
         <v>94</v>
       </c>
-      <c r="H11" s="32" t="n"/>
-      <c r="I11" s="30" t="n">
+      <c r="H11" s="30" t="n">
         <v>88</v>
       </c>
-      <c r="J11" s="33" t="n">
+      <c r="I11" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="33" t="n">
+      <c r="J11" s="32" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2679,17 +2662,16 @@
       <c r="F12" s="31" t="n">
         <v>63</v>
       </c>
-      <c r="G12" s="33" t="n">
+      <c r="G12" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="H12" s="32" t="n"/>
-      <c r="I12" s="33" t="n">
+      <c r="H12" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="J12" s="31" t="n">
+      <c r="I12" s="31" t="n">
         <v>66</v>
       </c>
-      <c r="K12" s="33" t="n">
+      <c r="J12" s="32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2702,7 +2684,7 @@
       <c r="B13" s="29" t="n">
         <v>59</v>
       </c>
-      <c r="C13" s="33" t="n">
+      <c r="C13" s="32" t="n">
         <v>22</v>
       </c>
       <c r="D13" s="30" t="n">
@@ -2717,14 +2699,13 @@
       <c r="G13" s="30" t="n">
         <v>92</v>
       </c>
-      <c r="H13" s="32" t="n"/>
-      <c r="I13" s="30" t="n">
+      <c r="H13" s="30" t="n">
         <v>82</v>
       </c>
-      <c r="J13" s="33" t="n">
+      <c r="I13" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="K13" s="33" t="n">
+      <c r="J13" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2740,26 +2721,25 @@
       <c r="C14" s="30" t="n">
         <v>72</v>
       </c>
-      <c r="D14" s="33" t="n">
+      <c r="D14" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="E14" s="33" t="n">
+      <c r="E14" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="33" t="n">
+      <c r="F14" s="32" t="n">
         <v>4</v>
       </c>
       <c r="G14" s="30" t="n">
         <v>82</v>
       </c>
-      <c r="H14" s="32" t="n"/>
+      <c r="H14" s="30" t="n">
+        <v>94</v>
+      </c>
       <c r="I14" s="30" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="J14" s="30" t="n">
-        <v>98</v>
-      </c>
-      <c r="K14" s="30" t="n">
         <v>86</v>
       </c>
     </row>
@@ -2772,10 +2752,10 @@
       <c r="B15" s="29" t="n">
         <v>58</v>
       </c>
-      <c r="C15" s="33" t="n">
+      <c r="C15" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="D15" s="33" t="n">
+      <c r="D15" s="32" t="n">
         <v>18</v>
       </c>
       <c r="E15" s="30" t="n">
@@ -2784,17 +2764,16 @@
       <c r="F15" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="G15" s="33" t="n">
+      <c r="G15" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="H15" s="32" t="n"/>
-      <c r="I15" s="31" t="n">
+      <c r="H15" s="31" t="n">
         <v>66</v>
       </c>
-      <c r="J15" s="33" t="n">
+      <c r="I15" s="32" t="n">
         <v>48</v>
       </c>
-      <c r="K15" s="33" t="n">
+      <c r="J15" s="32" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2807,7 +2786,7 @@
       <c r="B16" s="29" t="n">
         <v>57</v>
       </c>
-      <c r="C16" s="33" t="n">
+      <c r="C16" s="32" t="n">
         <v>36</v>
       </c>
       <c r="D16" s="31" t="n">
@@ -2822,14 +2801,13 @@
       <c r="G16" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="H16" s="32" t="n"/>
-      <c r="I16" s="30" t="n">
+      <c r="H16" s="30" t="n">
         <v>96</v>
       </c>
-      <c r="J16" s="32" t="n">
+      <c r="I16" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="31" t="n">
+      <c r="J16" s="31" t="n">
         <v>64</v>
       </c>
     </row>
@@ -2848,23 +2826,22 @@
       <c r="D17" s="30" t="n">
         <v>90</v>
       </c>
-      <c r="E17" s="33" t="n">
+      <c r="E17" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="F17" s="33" t="n">
+      <c r="F17" s="32" t="n">
         <v>24</v>
       </c>
       <c r="G17" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="H17" s="32" t="n"/>
+      <c r="H17" s="31" t="n">
+        <v>68</v>
+      </c>
       <c r="I17" s="31" t="n">
         <v>68</v>
       </c>
-      <c r="J17" s="31" t="n">
-        <v>68</v>
-      </c>
-      <c r="K17" s="33" t="n">
+      <c r="J17" s="32" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2880,26 +2857,25 @@
       <c r="C18" s="30" t="n">
         <v>96</v>
       </c>
-      <c r="D18" s="33" t="n">
+      <c r="D18" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="E18" s="33" t="n">
+      <c r="E18" s="32" t="n">
         <v>48</v>
       </c>
-      <c r="F18" s="33" t="n">
+      <c r="F18" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="G18" s="33" t="n">
+      <c r="G18" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="H18" s="32" t="n"/>
-      <c r="I18" s="31" t="n">
+      <c r="H18" s="31" t="n">
         <v>52</v>
       </c>
-      <c r="J18" s="33" t="n">
+      <c r="I18" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="K18" s="30" t="n">
+      <c r="J18" s="30" t="n">
         <v>82</v>
       </c>
     </row>
@@ -2915,26 +2891,25 @@
       <c r="C19" s="31" t="n">
         <v>64</v>
       </c>
-      <c r="D19" s="33" t="n">
+      <c r="D19" s="32" t="n">
         <v>14</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>84</v>
       </c>
-      <c r="F19" s="33" t="n">
+      <c r="F19" s="32" t="n">
         <v>18</v>
       </c>
       <c r="G19" s="31" t="n">
         <v>58</v>
       </c>
-      <c r="H19" s="32" t="n"/>
-      <c r="I19" s="33" t="n">
+      <c r="H19" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="J19" s="30" t="n">
+      <c r="I19" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="K19" s="33" t="n">
+      <c r="J19" s="32" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2947,7 +2922,7 @@
       <c r="B20" s="29" t="n">
         <v>50</v>
       </c>
-      <c r="C20" s="33" t="n">
+      <c r="C20" s="32" t="n">
         <v>14</v>
       </c>
       <c r="D20" s="31" t="n">
@@ -2962,14 +2937,13 @@
       <c r="G20" s="30" t="n">
         <v>74</v>
       </c>
-      <c r="H20" s="32" t="n"/>
-      <c r="I20" s="31" t="n">
+      <c r="H20" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="J20" s="33" t="n">
+      <c r="I20" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="K20" s="33" t="n">
+      <c r="J20" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2985,26 +2959,25 @@
       <c r="C21" s="31" t="n">
         <v>58</v>
       </c>
-      <c r="D21" s="33" t="n">
+      <c r="D21" s="32" t="n">
         <v>20</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>94</v>
       </c>
-      <c r="F21" s="33" t="n">
+      <c r="F21" s="32" t="n">
         <v>12</v>
       </c>
       <c r="G21" s="30" t="n">
         <v>70</v>
       </c>
-      <c r="H21" s="32" t="n"/>
-      <c r="I21" s="31" t="n">
+      <c r="H21" s="31" t="n">
         <v>54</v>
       </c>
-      <c r="J21" s="33" t="n">
+      <c r="I21" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="K21" s="30" t="n">
+      <c r="J21" s="30" t="n">
         <v>70</v>
       </c>
     </row>
@@ -3029,17 +3002,16 @@
       <c r="F22" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="G22" s="33" t="n">
+      <c r="G22" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="H22" s="32" t="n"/>
-      <c r="I22" s="33" t="n">
+      <c r="H22" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="J22" s="33" t="n">
+      <c r="I22" s="32" t="n">
         <v>44</v>
       </c>
-      <c r="K22" s="30" t="n">
+      <c r="J22" s="30" t="n">
         <v>88</v>
       </c>
     </row>
@@ -3058,23 +3030,22 @@
       <c r="D23" s="30" t="n">
         <v>73</v>
       </c>
-      <c r="E23" s="33" t="n">
+      <c r="E23" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="F23" s="32" t="n">
+      <c r="F23" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="31" t="n">
         <v>66</v>
       </c>
-      <c r="H23" s="32" t="n"/>
-      <c r="I23" s="31" t="n">
+      <c r="H23" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="J23" s="30" t="n">
+      <c r="I23" s="30" t="n">
         <v>82</v>
       </c>
-      <c r="K23" s="33" t="n">
+      <c r="J23" s="32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3087,29 +3058,28 @@
       <c r="B24" s="29" t="n">
         <v>49</v>
       </c>
-      <c r="C24" s="33" t="n">
+      <c r="C24" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="D24" s="33" t="n">
+      <c r="D24" s="32" t="n">
         <v>27</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>88</v>
       </c>
-      <c r="F24" s="33" t="n">
+      <c r="F24" s="32" t="n">
         <v>39</v>
       </c>
       <c r="G24" s="30" t="n">
         <v>72</v>
       </c>
-      <c r="H24" s="32" t="n"/>
-      <c r="I24" s="33" t="n">
+      <c r="H24" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="J24" s="30" t="n">
+      <c r="I24" s="30" t="n">
         <v>94</v>
       </c>
-      <c r="K24" s="31" t="n">
+      <c r="J24" s="31" t="n">
         <v>60</v>
       </c>
     </row>
@@ -3122,29 +3092,28 @@
       <c r="B25" s="29" t="n">
         <v>49</v>
       </c>
-      <c r="C25" s="33" t="n">
+      <c r="C25" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="D25" s="33" t="n">
+      <c r="D25" s="32" t="n">
         <v>39</v>
       </c>
-      <c r="E25" s="33" t="n">
+      <c r="E25" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="F25" s="33" t="n">
+      <c r="F25" s="32" t="n">
         <v>49</v>
       </c>
-      <c r="G25" s="33" t="n">
+      <c r="G25" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="H25" s="32" t="n"/>
+      <c r="H25" s="30" t="n">
+        <v>74</v>
+      </c>
       <c r="I25" s="30" t="n">
-        <v>74</v>
-      </c>
-      <c r="J25" s="30" t="n">
         <v>84</v>
       </c>
-      <c r="K25" s="33" t="n">
+      <c r="J25" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -3160,10 +3129,10 @@
       <c r="C26" s="31" t="n">
         <v>62</v>
       </c>
-      <c r="D26" s="33" t="n">
+      <c r="D26" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="E26" s="33" t="n">
+      <c r="E26" s="32" t="n">
         <v>28</v>
       </c>
       <c r="F26" s="31" t="n">
@@ -3172,14 +3141,13 @@
       <c r="G26" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="31" t="n">
+      <c r="H26" s="31" t="n">
         <v>58</v>
       </c>
-      <c r="J26" s="33" t="n">
+      <c r="I26" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="K26" s="30" t="n">
+      <c r="J26" s="30" t="n">
         <v>74</v>
       </c>
     </row>
@@ -3198,7 +3166,7 @@
       <c r="D27" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="E27" s="33" t="n">
+      <c r="E27" s="32" t="n">
         <v>4</v>
       </c>
       <c r="F27" s="31" t="n">
@@ -3207,14 +3175,13 @@
       <c r="G27" s="31" t="n">
         <v>62</v>
       </c>
-      <c r="H27" s="32" t="n"/>
-      <c r="I27" s="33" t="n">
+      <c r="H27" s="32" t="n">
         <v>36</v>
       </c>
+      <c r="I27" s="31" t="n">
+        <v>54</v>
+      </c>
       <c r="J27" s="31" t="n">
-        <v>54</v>
-      </c>
-      <c r="K27" s="31" t="n">
         <v>58</v>
       </c>
     </row>
@@ -3227,13 +3194,13 @@
       <c r="B28" s="29" t="n">
         <v>46</v>
       </c>
-      <c r="C28" s="33" t="n">
+      <c r="C28" s="32" t="n">
         <v>14</v>
       </c>
       <c r="D28" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="E28" s="33" t="n">
+      <c r="E28" s="32" t="n">
         <v>26</v>
       </c>
       <c r="F28" s="31" t="n">
@@ -3242,14 +3209,13 @@
       <c r="G28" s="30" t="n">
         <v>90</v>
       </c>
-      <c r="H28" s="32" t="n"/>
-      <c r="I28" s="30" t="n">
+      <c r="H28" s="30" t="n">
         <v>78</v>
       </c>
-      <c r="J28" s="33" t="n">
+      <c r="I28" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="K28" s="31" t="n">
+      <c r="J28" s="31" t="n">
         <v>52</v>
       </c>
     </row>
@@ -3262,10 +3228,10 @@
       <c r="B29" s="29" t="n">
         <v>46</v>
       </c>
-      <c r="C29" s="33" t="n">
+      <c r="C29" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="D29" s="33" t="n">
+      <c r="D29" s="32" t="n">
         <v>45</v>
       </c>
       <c r="E29" s="31" t="n">
@@ -3274,17 +3240,16 @@
       <c r="F29" s="30" t="n">
         <v>82</v>
       </c>
-      <c r="G29" s="33" t="n">
+      <c r="G29" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="32" t="n"/>
-      <c r="I29" s="33" t="n">
+      <c r="H29" s="32" t="n">
         <v>34</v>
       </c>
-      <c r="J29" s="33" t="n">
+      <c r="I29" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="K29" s="30" t="n">
+      <c r="J29" s="30" t="n">
         <v>80</v>
       </c>
     </row>
@@ -3297,29 +3262,28 @@
       <c r="B30" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="C30" s="33" t="n">
+      <c r="C30" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="D30" s="33" t="n">
+      <c r="D30" s="32" t="n">
         <v>4</v>
       </c>
       <c r="E30" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="F30" s="33" t="n">
+      <c r="F30" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="G30" s="33" t="n">
+      <c r="G30" s="32" t="n">
         <v>48</v>
       </c>
-      <c r="H30" s="32" t="n"/>
-      <c r="I30" s="30" t="n">
+      <c r="H30" s="30" t="n">
         <v>76</v>
       </c>
-      <c r="J30" s="33" t="n">
+      <c r="I30" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="K30" s="31" t="n">
+      <c r="J30" s="31" t="n">
         <v>68</v>
       </c>
     </row>
@@ -3335,7 +3299,7 @@
       <c r="C31" s="31" t="n">
         <v>52</v>
       </c>
-      <c r="D31" s="33" t="n">
+      <c r="D31" s="32" t="n">
         <v>10</v>
       </c>
       <c r="E31" s="30" t="n">
@@ -3344,17 +3308,16 @@
       <c r="F31" s="30" t="n">
         <v>73</v>
       </c>
-      <c r="G31" s="33" t="n">
+      <c r="G31" s="32" t="n">
         <v>34</v>
       </c>
-      <c r="H31" s="32" t="n"/>
-      <c r="I31" s="32" t="n">
+      <c r="H31" s="33" t="n">
         <v>0</v>
       </c>
+      <c r="I31" s="30" t="n">
+        <v>90</v>
+      </c>
       <c r="J31" s="30" t="n">
-        <v>90</v>
-      </c>
-      <c r="K31" s="30" t="n">
         <v>78</v>
       </c>
     </row>
@@ -3367,29 +3330,28 @@
       <c r="B32" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="C32" s="33" t="n">
+      <c r="C32" s="32" t="n">
         <v>34</v>
       </c>
       <c r="D32" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E32" s="33" t="n">
+      <c r="E32" s="32" t="n">
         <v>44</v>
       </c>
-      <c r="F32" s="33" t="n">
+      <c r="F32" s="32" t="n">
         <v>14</v>
       </c>
       <c r="G32" s="31" t="n">
         <v>52</v>
       </c>
-      <c r="H32" s="32" t="n"/>
-      <c r="I32" s="33" t="n">
+      <c r="H32" s="32" t="n">
         <v>18</v>
       </c>
+      <c r="I32" s="30" t="n">
+        <v>92</v>
+      </c>
       <c r="J32" s="30" t="n">
-        <v>92</v>
-      </c>
-      <c r="K32" s="30" t="n">
         <v>98</v>
       </c>
     </row>
@@ -3408,23 +3370,22 @@
       <c r="D33" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="E33" s="33" t="n">
+      <c r="E33" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="F33" s="33" t="n">
+      <c r="F33" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="G33" s="33" t="n">
+      <c r="G33" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="H33" s="32" t="n"/>
-      <c r="I33" s="33" t="n">
+      <c r="H33" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="J33" s="31" t="n">
+      <c r="I33" s="31" t="n">
         <v>64</v>
       </c>
-      <c r="K33" s="30" t="n">
+      <c r="J33" s="30" t="n">
         <v>92</v>
       </c>
     </row>
@@ -3437,13 +3398,13 @@
       <c r="B34" s="29" t="n">
         <v>41</v>
       </c>
-      <c r="C34" s="33" t="n">
+      <c r="C34" s="32" t="n">
         <v>6</v>
       </c>
       <c r="D34" s="31" t="n">
         <v>69</v>
       </c>
-      <c r="E34" s="33" t="n">
+      <c r="E34" s="32" t="n">
         <v>22</v>
       </c>
       <c r="F34" s="31" t="n">
@@ -3452,14 +3413,13 @@
       <c r="G34" s="30" t="n">
         <v>78</v>
       </c>
-      <c r="H34" s="32" t="n"/>
-      <c r="I34" s="31" t="n">
+      <c r="H34" s="31" t="n">
         <v>60</v>
       </c>
-      <c r="J34" s="33" t="n">
+      <c r="I34" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="K34" s="30" t="n">
+      <c r="J34" s="30" t="n">
         <v>76</v>
       </c>
     </row>
@@ -3472,29 +3432,28 @@
       <c r="B35" s="29" t="n">
         <v>41</v>
       </c>
-      <c r="C35" s="33" t="n">
+      <c r="C35" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="D35" s="33" t="n">
+      <c r="D35" s="32" t="n">
         <v>41</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>92</v>
       </c>
-      <c r="F35" s="33" t="n">
+      <c r="F35" s="32" t="n">
         <v>27</v>
       </c>
       <c r="G35" s="30" t="n">
         <v>76</v>
       </c>
-      <c r="H35" s="32" t="n"/>
-      <c r="I35" s="33" t="n">
+      <c r="H35" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="J35" s="33" t="n">
+      <c r="I35" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="K35" s="33" t="n">
+      <c r="J35" s="32" t="n">
         <v>28</v>
       </c>
     </row>
@@ -3510,26 +3469,25 @@
       <c r="C36" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="D36" s="33" t="n">
+      <c r="D36" s="32" t="n">
         <v>22</v>
       </c>
       <c r="E36" s="30" t="n">
         <v>78</v>
       </c>
-      <c r="F36" s="33" t="n">
+      <c r="F36" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="G36" s="33" t="n">
+      <c r="G36" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="H36" s="32" t="n"/>
-      <c r="I36" s="33" t="n">
+      <c r="H36" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="J36" s="30" t="n">
+      <c r="I36" s="30" t="n">
         <v>96</v>
       </c>
-      <c r="K36" s="33" t="n">
+      <c r="J36" s="32" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3542,13 +3500,13 @@
       <c r="B37" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="C37" s="33" t="n">
+      <c r="C37" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="33" t="n">
+      <c r="D37" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="E37" s="33" t="n">
+      <c r="E37" s="32" t="n">
         <v>34</v>
       </c>
       <c r="F37" s="31" t="n">
@@ -3557,14 +3515,13 @@
       <c r="G37" s="30" t="n">
         <v>84</v>
       </c>
-      <c r="H37" s="32" t="n"/>
-      <c r="I37" s="30" t="n">
+      <c r="H37" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="J37" s="33" t="n">
+      <c r="I37" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="K37" s="33" t="n">
+      <c r="J37" s="32" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3577,29 +3534,28 @@
       <c r="B38" s="29" t="n">
         <v>38</v>
       </c>
-      <c r="C38" s="33" t="n">
+      <c r="C38" s="32" t="n">
         <v>28</v>
       </c>
       <c r="D38" s="30" t="n">
         <v>82</v>
       </c>
-      <c r="E38" s="33" t="n">
+      <c r="E38" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="F38" s="33" t="n">
+      <c r="F38" s="32" t="n">
         <v>2</v>
       </c>
       <c r="G38" s="31" t="n">
         <v>68</v>
       </c>
-      <c r="H38" s="32" t="n"/>
-      <c r="I38" s="33" t="n">
+      <c r="H38" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="J38" s="33" t="n">
+      <c r="I38" s="32" t="n">
         <v>34</v>
       </c>
-      <c r="K38" s="33" t="n">
+      <c r="J38" s="32" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3612,29 +3568,28 @@
       <c r="B39" s="29" t="n">
         <v>37</v>
       </c>
-      <c r="C39" s="33" t="n">
+      <c r="C39" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="D39" s="33" t="n">
+      <c r="D39" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="E39" s="33" t="n">
+      <c r="E39" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="F39" s="33" t="n">
+      <c r="F39" s="32" t="n">
         <v>29</v>
       </c>
-      <c r="G39" s="33" t="n">
+      <c r="G39" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="H39" s="32" t="n"/>
+      <c r="H39" s="31" t="n">
+        <v>64</v>
+      </c>
       <c r="I39" s="31" t="n">
-        <v>64</v>
-      </c>
-      <c r="J39" s="31" t="n">
         <v>62</v>
       </c>
-      <c r="K39" s="33" t="n">
+      <c r="J39" s="32" t="n">
         <v>30</v>
       </c>
     </row>
@@ -3647,29 +3602,28 @@
       <c r="B40" s="29" t="n">
         <v>37</v>
       </c>
-      <c r="C40" s="32" t="n">
+      <c r="C40" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="33" t="n">
+      <c r="D40" s="32" t="n">
         <v>12</v>
       </c>
       <c r="E40" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="F40" s="33" t="n">
+      <c r="F40" s="32" t="n">
         <v>45</v>
       </c>
-      <c r="G40" s="33" t="n">
+      <c r="G40" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="H40" s="32" t="n"/>
-      <c r="I40" s="33" t="n">
+      <c r="H40" s="32" t="n">
         <v>44</v>
       </c>
-      <c r="J40" s="33" t="n">
+      <c r="I40" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="K40" s="31" t="n">
+      <c r="J40" s="31" t="n">
         <v>54</v>
       </c>
     </row>
@@ -3682,29 +3636,28 @@
       <c r="B41" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="C41" s="33" t="n">
+      <c r="C41" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="D41" s="33" t="n">
+      <c r="D41" s="32" t="n">
         <v>8</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>86</v>
       </c>
-      <c r="F41" s="33" t="n">
+      <c r="F41" s="32" t="n">
         <v>41</v>
       </c>
-      <c r="G41" s="32" t="n">
+      <c r="G41" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="32" t="n"/>
-      <c r="I41" s="33" t="n">
+      <c r="H41" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="J41" s="33" t="n">
+      <c r="I41" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="K41" s="33" t="n">
+      <c r="J41" s="32" t="n">
         <v>44</v>
       </c>
     </row>
@@ -3717,10 +3670,10 @@
       <c r="B42" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="C42" s="33" t="n">
+      <c r="C42" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="D42" s="33" t="n">
+      <c r="D42" s="32" t="n">
         <v>29</v>
       </c>
       <c r="E42" s="30" t="n">
@@ -3729,19 +3682,18 @@
       <c r="F42" s="31" t="n">
         <v>67</v>
       </c>
-      <c r="G42" s="33" t="n">
+      <c r="G42" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="H42" s="32" t="n"/>
-      <c r="I42" s="32" t="n">
+      <c r="H42" s="33" t="n">
         <v>0</v>
+      </c>
+      <c r="I42" s="31" t="n">
+        <v>56</v>
       </c>
       <c r="J42" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="K42" s="31" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3752,13 +3704,13 @@
       <c r="B43" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="C43" s="33" t="n">
+      <c r="C43" s="32" t="n">
         <v>18</v>
       </c>
       <c r="D43" s="31" t="n">
         <v>67</v>
       </c>
-      <c r="E43" s="33" t="n">
+      <c r="E43" s="32" t="n">
         <v>2</v>
       </c>
       <c r="F43" s="31" t="n">
@@ -3767,14 +3719,13 @@
       <c r="G43" s="31" t="n">
         <v>54</v>
       </c>
-      <c r="H43" s="32" t="n"/>
-      <c r="I43" s="33" t="n">
+      <c r="H43" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="J43" s="30" t="n">
+      <c r="I43" s="30" t="n">
         <v>70</v>
       </c>
-      <c r="K43" s="33" t="n">
+      <c r="J43" s="32" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3787,13 +3738,13 @@
       <c r="B44" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="C44" s="33" t="n">
+      <c r="C44" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D44" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="E44" s="33" t="n">
+      <c r="E44" s="32" t="n">
         <v>20</v>
       </c>
       <c r="F44" s="30" t="n">
@@ -3802,14 +3753,13 @@
       <c r="G44" s="31" t="n">
         <v>60</v>
       </c>
-      <c r="H44" s="32" t="n"/>
-      <c r="I44" s="33" t="n">
+      <c r="H44" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="J44" s="31" t="n">
+      <c r="I44" s="31" t="n">
         <v>58</v>
       </c>
-      <c r="K44" s="33" t="n">
+      <c r="J44" s="32" t="n">
         <v>42</v>
       </c>
     </row>
@@ -3828,23 +3778,22 @@
       <c r="D45" s="31" t="n">
         <v>51</v>
       </c>
-      <c r="E45" s="32" t="n">
+      <c r="E45" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="33" t="n">
+      <c r="F45" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="G45" s="33" t="n">
+      <c r="G45" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="H45" s="32" t="n"/>
-      <c r="I45" s="33" t="n">
+      <c r="H45" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="J45" s="31" t="n">
+      <c r="I45" s="31" t="n">
         <v>52</v>
       </c>
-      <c r="K45" s="30" t="n">
+      <c r="J45" s="30" t="n">
         <v>90</v>
       </c>
     </row>
@@ -3857,29 +3806,28 @@
       <c r="B46" s="29" t="n">
         <v>32</v>
       </c>
-      <c r="C46" s="33" t="n">
+      <c r="C46" s="32" t="n">
         <v>48</v>
       </c>
-      <c r="D46" s="33" t="n">
+      <c r="D46" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="E46" s="33" t="n">
+      <c r="E46" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="F46" s="33" t="n">
+      <c r="F46" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="G46" s="33" t="n">
+      <c r="G46" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="H46" s="32" t="n"/>
-      <c r="I46" s="33" t="n">
+      <c r="H46" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="J46" s="30" t="n">
+      <c r="I46" s="30" t="n">
         <v>74</v>
       </c>
-      <c r="K46" s="33" t="n">
+      <c r="J46" s="32" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3895,26 +3843,25 @@
       <c r="C47" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="D47" s="33" t="n">
+      <c r="D47" s="32" t="n">
         <v>31</v>
       </c>
-      <c r="E47" s="33" t="n">
+      <c r="E47" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="F47" s="33" t="n">
+      <c r="F47" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="G47" s="33" t="n">
+      <c r="G47" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="H47" s="32" t="n"/>
-      <c r="I47" s="33" t="n">
+      <c r="H47" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="J47" s="31" t="n">
+      <c r="I47" s="31" t="n">
         <v>60</v>
       </c>
-      <c r="K47" s="32" t="n">
+      <c r="J47" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3927,29 +3874,28 @@
       <c r="B48" s="29" t="n">
         <v>29</v>
       </c>
-      <c r="C48" s="33" t="n">
+      <c r="C48" s="32" t="n">
         <v>2</v>
       </c>
       <c r="D48" s="30" t="n">
         <v>94</v>
       </c>
-      <c r="E48" s="33" t="n">
+      <c r="E48" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="F48" s="33" t="n">
+      <c r="F48" s="32" t="n">
         <v>31</v>
       </c>
-      <c r="G48" s="33" t="n">
+      <c r="G48" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="H48" s="32" t="n"/>
-      <c r="I48" s="33" t="n">
+      <c r="H48" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="J48" s="33" t="n">
+      <c r="I48" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="K48" s="30" t="n">
+      <c r="J48" s="30" t="n">
         <v>84</v>
       </c>
     </row>
@@ -3962,29 +3908,28 @@
       <c r="B49" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="C49" s="33" t="n">
+      <c r="C49" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="D49" s="33" t="n">
+      <c r="D49" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="E49" s="33" t="n">
+      <c r="E49" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="F49" s="33" t="n">
+      <c r="F49" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="G49" s="33" t="n">
+      <c r="G49" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="H49" s="32" t="n"/>
-      <c r="I49" s="33" t="n">
+      <c r="H49" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="J49" s="33" t="n">
+      <c r="I49" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="K49" s="33" t="n">
+      <c r="J49" s="32" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4000,26 +3945,25 @@
       <c r="C50" s="30" t="n">
         <v>70</v>
       </c>
-      <c r="D50" s="32" t="n">
+      <c r="D50" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="E50" s="33" t="n">
+      <c r="E50" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="F50" s="33" t="n">
+      <c r="F50" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="G50" s="33" t="n">
+      <c r="G50" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="H50" s="32" t="n"/>
-      <c r="I50" s="33" t="n">
+      <c r="H50" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="J50" s="33" t="n">
+      <c r="I50" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="K50" s="33" t="n">
+      <c r="J50" s="32" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4032,29 +3976,28 @@
       <c r="B51" s="29" t="n">
         <v>18</v>
       </c>
-      <c r="C51" s="33" t="n">
+      <c r="C51" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="D51" s="33" t="n">
+      <c r="D51" s="32" t="n">
         <v>47</v>
       </c>
-      <c r="E51" s="33" t="n">
+      <c r="E51" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="F51" s="33" t="n">
+      <c r="F51" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="G51" s="33" t="n">
+      <c r="G51" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="H51" s="32" t="n"/>
-      <c r="I51" s="33" t="n">
+      <c r="H51" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="J51" s="33" t="n">
+      <c r="I51" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="K51" s="30" t="n">
+      <c r="J51" s="30" t="n">
         <v>72</v>
       </c>
     </row>
@@ -4165,35 +4108,35 @@
           <t>80 (A+)</t>
         </is>
       </c>
-      <c r="C2" s="32" t="n">
+      <c r="C2" s="33" t="n">
         <v>3.1</v>
       </c>
-      <c r="D2" s="32" t="n">
+      <c r="D2" s="33" t="n">
         <v>0.37</v>
       </c>
-      <c r="E2" s="32" t="n">
+      <c r="E2" s="33" t="n">
         <v>3.78</v>
       </c>
-      <c r="F2" s="32" t="n">
+      <c r="F2" s="33" t="n">
         <v>1.49</v>
       </c>
-      <c r="G2" s="32" t="n">
+      <c r="G2" s="33" t="n">
         <v>4.54</v>
       </c>
-      <c r="H2" s="32" t="n"/>
-      <c r="I2" s="32" t="n">
+      <c r="H2" s="33" t="n"/>
+      <c r="I2" s="33" t="n">
         <v>2.64</v>
       </c>
-      <c r="J2" s="32" t="n">
+      <c r="J2" s="33" t="n">
         <v>31.25</v>
       </c>
-      <c r="K2" s="32" t="n">
+      <c r="K2" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L2" s="32" t="n">
+      <c r="L2" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="32" t="n">
+      <c r="M2" s="33" t="n">
         <v>50</v>
       </c>
     </row>
@@ -4208,35 +4151,35 @@
           <t>77 (A+)</t>
         </is>
       </c>
-      <c r="C3" s="32" t="n">
+      <c r="C3" s="33" t="n">
         <v>2.7</v>
       </c>
-      <c r="D3" s="32" t="n">
+      <c r="D3" s="33" t="n">
         <v>2.77</v>
       </c>
-      <c r="E3" s="32" t="n">
+      <c r="E3" s="33" t="n">
         <v>4.73</v>
       </c>
-      <c r="F3" s="32" t="n">
+      <c r="F3" s="33" t="n">
         <v>1.9</v>
       </c>
-      <c r="G3" s="32" t="n">
+      <c r="G3" s="33" t="n">
         <v>2.14</v>
       </c>
-      <c r="H3" s="32" t="n"/>
-      <c r="I3" s="32" t="n">
+      <c r="H3" s="33" t="n"/>
+      <c r="I3" s="33" t="n">
         <v>1.88</v>
       </c>
-      <c r="J3" s="32" t="n">
+      <c r="J3" s="33" t="n">
         <v>18.05</v>
       </c>
-      <c r="K3" s="32" t="n">
+      <c r="K3" s="33" t="n">
         <v>6.16</v>
       </c>
-      <c r="L3" s="32" t="n">
+      <c r="L3" s="33" t="n">
         <v>3.57</v>
       </c>
-      <c r="M3" s="32" t="n">
+      <c r="M3" s="33" t="n">
         <v>29</v>
       </c>
     </row>
@@ -4251,35 +4194,35 @@
           <t>75 (A+)</t>
         </is>
       </c>
-      <c r="C4" s="32" t="n">
+      <c r="C4" s="33" t="n">
         <v>3.6</v>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="33" t="n">
         <v>0.33</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="33" t="n">
         <v>4.7</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="33" t="n">
         <v>1.52</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="33" t="n">
         <v>3.28</v>
       </c>
-      <c r="H4" s="32" t="n"/>
-      <c r="I4" s="32" t="n">
+      <c r="H4" s="33" t="n"/>
+      <c r="I4" s="33" t="n">
         <v>1.57</v>
       </c>
-      <c r="J4" s="32" t="n">
+      <c r="J4" s="33" t="n">
         <v>-5.1</v>
       </c>
-      <c r="K4" s="32" t="n">
+      <c r="K4" s="33" t="n">
         <v>7.38</v>
       </c>
-      <c r="L4" s="32" t="n">
+      <c r="L4" s="33" t="n">
         <v>6.25</v>
       </c>
-      <c r="M4" s="32" t="n">
+      <c r="M4" s="33" t="n">
         <v>51</v>
       </c>
     </row>
@@ -4294,35 +4237,35 @@
           <t>74 (A+)</t>
         </is>
       </c>
-      <c r="C5" s="32" t="n">
+      <c r="C5" s="33" t="n">
         <v>3.9</v>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="33" t="n">
         <v>0.14</v>
       </c>
-      <c r="E5" s="32" t="n">
+      <c r="E5" s="33" t="n">
         <v>6.37</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="33" t="n">
         <v>1.29</v>
       </c>
-      <c r="G5" s="32" t="n">
+      <c r="G5" s="33" t="n">
         <v>2.18</v>
       </c>
-      <c r="H5" s="32" t="n"/>
-      <c r="I5" s="32" t="n">
+      <c r="H5" s="33" t="n"/>
+      <c r="I5" s="33" t="n">
         <v>1.08</v>
       </c>
-      <c r="J5" s="32" t="n">
+      <c r="J5" s="33" t="n">
         <v>47.86</v>
       </c>
-      <c r="K5" s="32" t="n">
+      <c r="K5" s="33" t="n">
         <v>8.56</v>
       </c>
-      <c r="L5" s="32" t="n">
+      <c r="L5" s="33" t="n">
         <v>15.62</v>
       </c>
-      <c r="M5" s="32" t="n">
+      <c r="M5" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -4337,35 +4280,35 @@
           <t>73 (A+)</t>
         </is>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="33" t="n">
         <v>3.7</v>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="33" t="n">
         <v>7.7</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>1.35</v>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="33" t="n">
         <v>1.68</v>
       </c>
-      <c r="H6" s="32" t="n"/>
-      <c r="I6" s="32" t="n">
+      <c r="H6" s="33" t="n"/>
+      <c r="I6" s="33" t="n">
         <v>0.84</v>
       </c>
-      <c r="J6" s="32" t="n">
+      <c r="J6" s="33" t="n">
         <v>-1.26</v>
       </c>
-      <c r="K6" s="32" t="n">
+      <c r="K6" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L6" s="32" t="n">
+      <c r="L6" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="32" t="n">
+      <c r="M6" s="33" t="n">
         <v>45</v>
       </c>
     </row>
@@ -4380,35 +4323,35 @@
           <t>71 (A+)</t>
         </is>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="33" t="n">
         <v>3.3</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <v>-0.14</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>5.97</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>2.14</v>
       </c>
-      <c r="G7" s="32" t="n">
+      <c r="G7" s="33" t="n">
         <v>3.92</v>
       </c>
-      <c r="H7" s="32" t="n"/>
-      <c r="I7" s="32" t="n">
+      <c r="H7" s="33" t="n"/>
+      <c r="I7" s="33" t="n">
         <v>1.56</v>
       </c>
-      <c r="J7" s="32" t="n">
+      <c r="J7" s="33" t="n">
         <v>-5.1</v>
       </c>
-      <c r="K7" s="32" t="n">
+      <c r="K7" s="33" t="n">
         <v>7.09</v>
       </c>
-      <c r="L7" s="32" t="n">
+      <c r="L7" s="33" t="n">
         <v>1.92</v>
       </c>
-      <c r="M7" s="32" t="n">
+      <c r="M7" s="33" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4423,35 +4366,35 @@
           <t>68 (A+)</t>
         </is>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="33" t="n">
         <v>3.6</v>
       </c>
-      <c r="D8" s="32" t="n">
+      <c r="D8" s="33" t="n">
         <v>0.96</v>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="33" t="n">
         <v>4.19</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="33" t="n">
         <v>2.28</v>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="33" t="n">
         <v>4.4</v>
       </c>
-      <c r="H8" s="32" t="n"/>
-      <c r="I8" s="32" t="n">
+      <c r="H8" s="33" t="n"/>
+      <c r="I8" s="33" t="n">
         <v>2.73</v>
       </c>
-      <c r="J8" s="32" t="n">
+      <c r="J8" s="33" t="n">
         <v>-21.89</v>
       </c>
-      <c r="K8" s="32" t="n">
+      <c r="K8" s="33" t="n">
         <v>7.28</v>
       </c>
-      <c r="L8" s="32" t="n">
+      <c r="L8" s="33" t="n">
         <v>4.17</v>
       </c>
-      <c r="M8" s="32" t="n">
+      <c r="M8" s="33" t="n">
         <v>50</v>
       </c>
     </row>
@@ -4466,35 +4409,35 @@
           <t>65 (A)</t>
         </is>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>3.8</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="33" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E9" s="32" t="n">
+      <c r="E9" s="33" t="n">
         <v>2.03</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="33" t="n">
         <v>1.72</v>
       </c>
-      <c r="G9" s="32" t="n">
+      <c r="G9" s="33" t="n">
         <v>2.18</v>
       </c>
-      <c r="H9" s="32" t="n"/>
-      <c r="I9" s="32" t="n">
+      <c r="H9" s="33" t="n"/>
+      <c r="I9" s="33" t="n">
         <v>0.44</v>
       </c>
-      <c r="J9" s="32" t="n">
+      <c r="J9" s="33" t="n">
         <v>16.2</v>
       </c>
-      <c r="K9" s="32" t="n">
+      <c r="K9" s="33" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="32" t="n">
+      <c r="L9" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="M9" s="32" t="n">
+      <c r="M9" s="33" t="n">
         <v>44</v>
       </c>
     </row>
@@ -4509,35 +4452,35 @@
           <t>64 (A)</t>
         </is>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>3.5</v>
       </c>
-      <c r="D10" s="32" t="n">
+      <c r="D10" s="33" t="n">
         <v>1.93</v>
       </c>
-      <c r="E10" s="32" t="n">
+      <c r="E10" s="33" t="n">
         <v>3.15</v>
       </c>
-      <c r="F10" s="32" t="n">
+      <c r="F10" s="33" t="n">
         <v>2.57</v>
       </c>
-      <c r="G10" s="32" t="n">
+      <c r="G10" s="33" t="n">
         <v>3.06</v>
       </c>
-      <c r="H10" s="32" t="n"/>
-      <c r="I10" s="32" t="n">
+      <c r="H10" s="33" t="n"/>
+      <c r="I10" s="33" t="n">
         <v>0.41</v>
       </c>
-      <c r="J10" s="32" t="n">
+      <c r="J10" s="33" t="n">
         <v>15.16</v>
       </c>
-      <c r="K10" s="32" t="n">
+      <c r="K10" s="33" t="n">
         <v>7.1</v>
       </c>
-      <c r="L10" s="32" t="n">
+      <c r="L10" s="33" t="n">
         <v>1.96</v>
       </c>
-      <c r="M10" s="32" t="n">
+      <c r="M10" s="33" t="n">
         <v>52</v>
       </c>
     </row>
@@ -4552,35 +4495,35 @@
           <t>62 (A-)</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="33" t="n">
         <v>4.1</v>
       </c>
-      <c r="D11" s="32" t="n">
+      <c r="D11" s="33" t="n">
         <v>1.27</v>
       </c>
-      <c r="E11" s="32" t="n">
+      <c r="E11" s="33" t="n">
         <v>4.74</v>
       </c>
-      <c r="F11" s="32" t="n">
+      <c r="F11" s="33" t="n">
         <v>1.02</v>
       </c>
-      <c r="G11" s="32" t="n">
+      <c r="G11" s="33" t="n">
         <v>4.22</v>
       </c>
-      <c r="H11" s="32" t="n"/>
-      <c r="I11" s="32" t="n">
+      <c r="H11" s="33" t="n"/>
+      <c r="I11" s="33" t="n">
         <v>1.89</v>
       </c>
-      <c r="J11" s="32" t="n">
+      <c r="J11" s="33" t="n">
         <v>-37.8</v>
       </c>
-      <c r="K11" s="32" t="n">
+      <c r="K11" s="33" t="n">
         <v>6.83</v>
       </c>
-      <c r="L11" s="32" t="n">
+      <c r="L11" s="33" t="n">
         <v>8.619999999999999</v>
       </c>
-      <c r="M11" s="32" t="n">
+      <c r="M11" s="33" t="n">
         <v>63</v>
       </c>
     </row>
@@ -4595,35 +4538,35 @@
           <t>60 (A-)</t>
         </is>
       </c>
-      <c r="C12" s="32" t="n">
+      <c r="C12" s="33" t="n">
         <v>3.8</v>
       </c>
-      <c r="D12" s="32" t="n">
+      <c r="D12" s="33" t="n">
         <v>2.55</v>
       </c>
-      <c r="E12" s="32" t="n">
+      <c r="E12" s="33" t="n">
         <v>5.61</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F12" s="33" t="n">
         <v>2.12</v>
       </c>
-      <c r="G12" s="32" t="n">
+      <c r="G12" s="33" t="n">
         <v>2.02</v>
       </c>
-      <c r="H12" s="32" t="n"/>
-      <c r="I12" s="32" t="n">
+      <c r="H12" s="33" t="n"/>
+      <c r="I12" s="33" t="n">
         <v>0.06</v>
       </c>
-      <c r="J12" s="32" t="n">
+      <c r="J12" s="33" t="n">
         <v>13.14</v>
       </c>
-      <c r="K12" s="32" t="n">
+      <c r="K12" s="33" t="n">
         <v>6.82</v>
       </c>
-      <c r="L12" s="32" t="n">
+      <c r="L12" s="33" t="n">
         <v>-2.08</v>
       </c>
-      <c r="M12" s="32" t="n">
+      <c r="M12" s="33" t="n">
         <v>47</v>
       </c>
     </row>
@@ -4638,35 +4581,35 @@
           <t>59 (B+)</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
+      <c r="C13" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="D13" s="32" t="n">
+      <c r="D13" s="33" t="n">
         <v>1.74</v>
       </c>
-      <c r="E13" s="32" t="n">
+      <c r="E13" s="33" t="n">
         <v>5.04</v>
       </c>
-      <c r="F13" s="32" t="n">
+      <c r="F13" s="33" t="n">
         <v>1.67</v>
       </c>
-      <c r="G13" s="32" t="n">
+      <c r="G13" s="33" t="n">
         <v>4.08</v>
       </c>
-      <c r="H13" s="32" t="n"/>
-      <c r="I13" s="32" t="n">
+      <c r="H13" s="33" t="n"/>
+      <c r="I13" s="33" t="n">
         <v>1.39</v>
       </c>
-      <c r="J13" s="32" t="n">
+      <c r="J13" s="33" t="n">
         <v>-17.79</v>
       </c>
-      <c r="K13" s="32" t="n">
+      <c r="K13" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L13" s="32" t="n">
+      <c r="L13" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="32" t="n">
+      <c r="M13" s="33" t="n">
         <v>70</v>
       </c>
     </row>
@@ -4681,35 +4624,35 @@
           <t>59 (A-)</t>
         </is>
       </c>
-      <c r="C14" s="32" t="n">
+      <c r="C14" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="32" t="n">
+      <c r="D14" s="33" t="n">
         <v>-0.6</v>
       </c>
-      <c r="E14" s="32" t="n">
+      <c r="E14" s="33" t="n">
         <v>0.27</v>
       </c>
-      <c r="F14" s="32" t="n">
+      <c r="F14" s="33" t="n">
         <v>6.19</v>
       </c>
-      <c r="G14" s="32" t="n">
+      <c r="G14" s="33" t="n">
         <v>3.4</v>
       </c>
-      <c r="H14" s="32" t="n"/>
-      <c r="I14" s="32" t="n">
+      <c r="H14" s="33" t="n"/>
+      <c r="I14" s="33" t="n">
         <v>1.44</v>
       </c>
-      <c r="J14" s="32" t="n">
+      <c r="J14" s="33" t="n">
         <v>132.71</v>
       </c>
-      <c r="K14" s="32" t="n">
+      <c r="K14" s="33" t="n">
         <v>7.88</v>
       </c>
-      <c r="L14" s="32" t="n">
+      <c r="L14" s="33" t="n">
         <v>8.82</v>
       </c>
-      <c r="M14" s="32" t="n">
+      <c r="M14" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -4724,35 +4667,35 @@
           <t>58 (B+)</t>
         </is>
       </c>
-      <c r="C15" s="32" t="n">
+      <c r="C15" s="33" t="n">
         <v>4.8</v>
       </c>
-      <c r="D15" s="32" t="n">
+      <c r="D15" s="33" t="n">
         <v>-1.37</v>
       </c>
-      <c r="E15" s="32" t="n">
+      <c r="E15" s="33" t="n">
         <v>9.02</v>
       </c>
-      <c r="F15" s="32" t="n">
+      <c r="F15" s="33" t="n">
         <v>0.15</v>
       </c>
-      <c r="G15" s="32" t="n">
+      <c r="G15" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="H15" s="32" t="n"/>
-      <c r="I15" s="32" t="n">
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="J15" s="32" t="n">
+      <c r="J15" s="33" t="n">
         <v>-1.49</v>
       </c>
-      <c r="K15" s="32" t="n">
+      <c r="K15" s="33" t="n">
         <v>6.72</v>
       </c>
-      <c r="L15" s="32" t="n">
+      <c r="L15" s="33" t="n">
         <v>10.34</v>
       </c>
-      <c r="M15" s="32" t="n">
+      <c r="M15" s="33" t="n">
         <v>64</v>
       </c>
     </row>
@@ -4767,35 +4710,35 @@
           <t>57 (B+)</t>
         </is>
       </c>
-      <c r="C16" s="32" t="n">
+      <c r="C16" s="33" t="n">
         <v>5.2</v>
       </c>
-      <c r="D16" s="32" t="n">
+      <c r="D16" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="E16" s="32" t="n">
+      <c r="E16" s="33" t="n">
         <v>4.53</v>
       </c>
-      <c r="F16" s="32" t="n">
+      <c r="F16" s="33" t="n">
         <v>2.33</v>
       </c>
-      <c r="G16" s="32" t="n">
+      <c r="G16" s="33" t="n">
         <v>3.82</v>
       </c>
-      <c r="H16" s="32" t="n"/>
-      <c r="I16" s="32" t="n">
+      <c r="H16" s="33" t="n"/>
+      <c r="I16" s="33" t="n">
         <v>2.93</v>
       </c>
-      <c r="J16" s="32" t="n">
+      <c r="J16" s="33" t="n">
         <v>-38.98</v>
       </c>
-      <c r="K16" s="32" t="n">
+      <c r="K16" s="33" t="n">
         <v>7.33</v>
       </c>
-      <c r="L16" s="32" t="n">
+      <c r="L16" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="M16" s="32" t="n">
+      <c r="M16" s="33" t="n">
         <v>55</v>
       </c>
     </row>
@@ -4810,35 +4753,35 @@
           <t>54 (B)</t>
         </is>
       </c>
-      <c r="C17" s="32" t="n">
+      <c r="C17" s="33" t="n">
         <v>4.1</v>
       </c>
-      <c r="D17" s="32" t="n">
+      <c r="D17" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="32" t="n">
+      <c r="E17" s="33" t="n">
         <v>0.68</v>
       </c>
-      <c r="F17" s="32" t="n">
+      <c r="F17" s="33" t="n">
         <v>3.43</v>
       </c>
-      <c r="G17" s="32" t="n">
+      <c r="G17" s="33" t="n">
         <v>2.58</v>
       </c>
-      <c r="H17" s="32" t="n"/>
-      <c r="I17" s="32" t="n">
+      <c r="H17" s="33" t="n"/>
+      <c r="I17" s="33" t="n">
         <v>0.61</v>
       </c>
-      <c r="J17" s="32" t="n">
+      <c r="J17" s="33" t="n">
         <v>14.19</v>
       </c>
-      <c r="K17" s="32" t="n">
+      <c r="K17" s="33" t="n">
         <v>6.51</v>
       </c>
-      <c r="L17" s="32" t="n">
+      <c r="L17" s="33" t="n">
         <v>-4.88</v>
       </c>
-      <c r="M17" s="32" t="n">
+      <c r="M17" s="33" t="n">
         <v>39</v>
       </c>
     </row>
@@ -4853,35 +4796,35 @@
           <t>54 (B)</t>
         </is>
       </c>
-      <c r="C18" s="32" t="n">
+      <c r="C18" s="33" t="n">
         <v>3.3</v>
       </c>
-      <c r="D18" s="32" t="n">
+      <c r="D18" s="33" t="n">
         <v>-0.43</v>
       </c>
-      <c r="E18" s="32" t="n">
+      <c r="E18" s="33" t="n">
         <v>3.49</v>
       </c>
-      <c r="F18" s="32" t="n">
+      <c r="F18" s="33" t="n">
         <v>2.7</v>
       </c>
-      <c r="G18" s="32" t="n">
+      <c r="G18" s="33" t="n">
         <v>1.4</v>
       </c>
-      <c r="H18" s="32" t="n"/>
-      <c r="I18" s="32" t="n">
+      <c r="H18" s="33" t="n"/>
+      <c r="I18" s="33" t="n">
         <v>0.44</v>
       </c>
-      <c r="J18" s="32" t="n">
+      <c r="J18" s="33" t="n">
         <v>-25.53</v>
       </c>
-      <c r="K18" s="32" t="n">
+      <c r="K18" s="33" t="n">
         <v>7.83</v>
       </c>
-      <c r="L18" s="32" t="n">
+      <c r="L18" s="33" t="n">
         <v>8.33</v>
       </c>
-      <c r="M18" s="32" t="n">
+      <c r="M18" s="33" t="n">
         <v>39</v>
       </c>
     </row>
@@ -4896,35 +4839,35 @@
           <t>50 (B-)</t>
         </is>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>4.2</v>
       </c>
-      <c r="D19" s="32" t="n">
+      <c r="D19" s="33" t="n">
         <v>-1.59</v>
       </c>
-      <c r="E19" s="32" t="n">
+      <c r="E19" s="33" t="n">
         <v>6.15</v>
       </c>
-      <c r="F19" s="32" t="n">
+      <c r="F19" s="33" t="n">
         <v>4.21</v>
       </c>
-      <c r="G19" s="32" t="n">
+      <c r="G19" s="33" t="n">
         <v>2.88</v>
       </c>
-      <c r="H19" s="32" t="n"/>
-      <c r="I19" s="32" t="n">
+      <c r="H19" s="33" t="n"/>
+      <c r="I19" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="J19" s="32" t="n">
+      <c r="J19" s="33" t="n">
         <v>19.88</v>
       </c>
-      <c r="K19" s="32" t="n">
+      <c r="K19" s="33" t="n">
         <v>6.25</v>
       </c>
-      <c r="L19" s="32" t="n">
+      <c r="L19" s="33" t="n">
         <v>-7.5</v>
       </c>
-      <c r="M19" s="32" t="n">
+      <c r="M19" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -4939,35 +4882,35 @@
           <t>50 (B-)</t>
         </is>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="33" t="n">
         <v>4.7</v>
       </c>
-      <c r="D20" s="32" t="n">
+      <c r="D20" s="33" t="n">
         <v>0.52</v>
       </c>
-      <c r="E20" s="32" t="n">
+      <c r="E20" s="33" t="n">
         <v>5.58</v>
       </c>
-      <c r="F20" s="32" t="n">
+      <c r="F20" s="33" t="n">
         <v>1.37</v>
       </c>
-      <c r="G20" s="32" t="n">
+      <c r="G20" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="H20" s="32" t="n"/>
-      <c r="I20" s="32" t="n">
+      <c r="H20" s="33" t="n"/>
+      <c r="I20" s="33" t="n">
         <v>0.23</v>
       </c>
-      <c r="J20" s="32" t="n">
+      <c r="J20" s="33" t="n">
         <v>-9.949999999999999</v>
       </c>
-      <c r="K20" s="32" t="n">
+      <c r="K20" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L20" s="32" t="n">
+      <c r="L20" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M20" s="32" t="n">
+      <c r="M20" s="33" t="n">
         <v>68</v>
       </c>
     </row>
@@ -4982,35 +4925,35 @@
           <t>50 (B-)</t>
         </is>
       </c>
-      <c r="C21" s="32" t="n">
+      <c r="C21" s="33" t="n">
         <v>4.4</v>
       </c>
-      <c r="D21" s="32" t="n">
+      <c r="D21" s="33" t="n">
         <v>-1.3</v>
       </c>
-      <c r="E21" s="32" t="n">
+      <c r="E21" s="33" t="n">
         <v>7.2</v>
       </c>
-      <c r="F21" s="32" t="n">
+      <c r="F21" s="33" t="n">
         <v>4.77</v>
       </c>
-      <c r="G21" s="32" t="n">
+      <c r="G21" s="33" t="n">
         <v>3.16</v>
       </c>
-      <c r="H21" s="32" t="n"/>
-      <c r="I21" s="32" t="n">
+      <c r="H21" s="33" t="n"/>
+      <c r="I21" s="33" t="n">
         <v>1.07</v>
       </c>
-      <c r="J21" s="32" t="n">
+      <c r="J21" s="33" t="n">
         <v>-23.29</v>
       </c>
-      <c r="K21" s="32" t="n">
+      <c r="K21" s="33" t="n">
         <v>7.49</v>
       </c>
-      <c r="L21" s="32" t="n">
+      <c r="L21" s="33" t="n">
         <v>4.88</v>
       </c>
-      <c r="M21" s="32" t="n">
+      <c r="M21" s="33" t="n">
         <v>43</v>
       </c>
     </row>
@@ -5025,35 +4968,35 @@
           <t>50 (B-)</t>
         </is>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="32" t="n">
+      <c r="D22" s="33" t="n">
         <v>1.23</v>
       </c>
-      <c r="E22" s="32" t="n">
+      <c r="E22" s="33" t="n">
         <v>3.93</v>
       </c>
-      <c r="F22" s="32" t="n">
+      <c r="F22" s="33" t="n">
         <v>1.58</v>
       </c>
-      <c r="G22" s="32" t="n">
+      <c r="G22" s="33" t="n">
         <v>1.66</v>
       </c>
-      <c r="H22" s="32" t="n"/>
-      <c r="I22" s="32" t="n">
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n">
         <v>-0.37</v>
       </c>
-      <c r="J22" s="32" t="n">
+      <c r="J22" s="33" t="n">
         <v>-2.81</v>
       </c>
-      <c r="K22" s="32" t="n">
+      <c r="K22" s="33" t="n">
         <v>7.91</v>
       </c>
-      <c r="L22" s="32" t="n">
+      <c r="L22" s="33" t="n">
         <v>9.09</v>
       </c>
-      <c r="M22" s="32" t="n">
+      <c r="M22" s="33" t="n">
         <v>36</v>
       </c>
     </row>
@@ -5068,35 +5011,35 @@
           <t>49 (B-)</t>
         </is>
       </c>
-      <c r="C23" s="32" t="n">
+      <c r="C23" s="33" t="n">
         <v>4.5</v>
       </c>
-      <c r="D23" s="32" t="n">
+      <c r="D23" s="33" t="n">
         <v>1.23</v>
       </c>
-      <c r="E23" s="32" t="n">
+      <c r="E23" s="33" t="n">
         <v>2.82</v>
       </c>
-      <c r="F23" s="32" t="n">
+      <c r="F23" s="33" t="n">
         <v>7.51</v>
       </c>
-      <c r="G23" s="32" t="n">
+      <c r="G23" s="33" t="n">
         <v>3.08</v>
       </c>
-      <c r="H23" s="32" t="n"/>
-      <c r="I23" s="32" t="n">
+      <c r="H23" s="33" t="n"/>
+      <c r="I23" s="33" t="n">
         <v>0.68</v>
       </c>
-      <c r="J23" s="32" t="n">
+      <c r="J23" s="33" t="n">
         <v>22.6</v>
       </c>
-      <c r="K23" s="32" t="n">
+      <c r="K23" s="33" t="n">
         <v>6.65</v>
       </c>
-      <c r="L23" s="32" t="n">
+      <c r="L23" s="33" t="n">
         <v>-4.08</v>
       </c>
-      <c r="M23" s="32" t="n">
+      <c r="M23" s="33" t="n">
         <v>47</v>
       </c>
     </row>
@@ -5111,35 +5054,35 @@
           <t>49 (B-)</t>
         </is>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="32" t="n">
+      <c r="D24" s="33" t="n">
         <v>-0.96</v>
       </c>
-      <c r="E24" s="32" t="n">
+      <c r="E24" s="33" t="n">
         <v>6.37</v>
       </c>
-      <c r="F24" s="32" t="n">
+      <c r="F24" s="33" t="n">
         <v>2.79</v>
       </c>
-      <c r="G24" s="32" t="n">
+      <c r="G24" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="H24" s="32" t="n"/>
-      <c r="I24" s="32" t="n">
+      <c r="H24" s="33" t="n"/>
+      <c r="I24" s="33" t="n">
         <v>0.27</v>
       </c>
-      <c r="J24" s="32" t="n">
+      <c r="J24" s="33" t="n">
         <v>91.03</v>
       </c>
-      <c r="K24" s="32" t="n">
+      <c r="K24" s="33" t="n">
         <v>7.28</v>
       </c>
-      <c r="L24" s="32" t="n">
+      <c r="L24" s="33" t="n">
         <v>2.78</v>
       </c>
-      <c r="M24" s="32" t="n">
+      <c r="M24" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -5154,35 +5097,35 @@
           <t>49 (B-)</t>
         </is>
       </c>
-      <c r="C25" s="32" t="n">
+      <c r="C25" s="33" t="n">
         <v>3.7</v>
       </c>
-      <c r="D25" s="32" t="n">
+      <c r="D25" s="33" t="n">
         <v>-0.28</v>
       </c>
-      <c r="E25" s="32" t="n">
+      <c r="E25" s="33" t="n">
         <v>0.59</v>
       </c>
-      <c r="F25" s="32" t="n">
+      <c r="F25" s="33" t="n">
         <v>2.56</v>
       </c>
-      <c r="G25" s="32" t="n">
+      <c r="G25" s="33" t="n">
         <v>2.42</v>
       </c>
-      <c r="H25" s="32" t="n"/>
-      <c r="I25" s="32" t="n">
+      <c r="H25" s="33" t="n"/>
+      <c r="I25" s="33" t="n">
         <v>0.97</v>
       </c>
-      <c r="J25" s="32" t="n">
+      <c r="J25" s="33" t="n">
         <v>31.24</v>
       </c>
-      <c r="K25" s="32" t="n">
+      <c r="K25" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L25" s="32" t="n">
+      <c r="L25" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M25" s="32" t="n">
+      <c r="M25" s="33" t="n">
         <v>54</v>
       </c>
     </row>
@@ -5197,35 +5140,35 @@
           <t>48 (B-)</t>
         </is>
       </c>
-      <c r="C26" s="32" t="n">
+      <c r="C26" s="33" t="n">
         <v>3.9</v>
       </c>
-      <c r="D26" s="32" t="n">
+      <c r="D26" s="33" t="n">
         <v>-2.15</v>
       </c>
-      <c r="E26" s="32" t="n">
+      <c r="E26" s="33" t="n">
         <v>2.01</v>
       </c>
-      <c r="F26" s="32" t="n">
+      <c r="F26" s="33" t="n">
         <v>2.01</v>
       </c>
-      <c r="G26" s="32" t="n">
+      <c r="G26" s="33" t="n">
         <v>2.86</v>
       </c>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="32" t="n">
+      <c r="H26" s="33" t="n"/>
+      <c r="I26" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="J26" s="32" t="n">
+      <c r="J26" s="33" t="n">
         <v>-14.11</v>
       </c>
-      <c r="K26" s="32" t="n">
+      <c r="K26" s="33" t="n">
         <v>7.53</v>
       </c>
-      <c r="L26" s="32" t="n">
+      <c r="L26" s="33" t="n">
         <v>6.67</v>
       </c>
-      <c r="M26" s="32" t="n">
+      <c r="M26" s="33" t="n">
         <v>48</v>
       </c>
     </row>
@@ -5240,33 +5183,33 @@
           <t>47 (B-)</t>
         </is>
       </c>
-      <c r="C27" s="32" t="n">
+      <c r="C27" s="33" t="n">
         <v>3.4</v>
       </c>
-      <c r="D27" s="32" t="n">
+      <c r="D27" s="33" t="n">
         <v>1.8</v>
       </c>
-      <c r="E27" s="32" t="n">
+      <c r="E27" s="33" t="n">
         <v>-0.32</v>
       </c>
-      <c r="F27" s="32" t="n"/>
-      <c r="G27" s="32" t="n">
+      <c r="F27" s="33" t="n"/>
+      <c r="G27" s="33" t="n">
         <v>3.04</v>
       </c>
-      <c r="H27" s="32" t="n"/>
-      <c r="I27" s="32" t="n">
+      <c r="H27" s="33" t="n"/>
+      <c r="I27" s="33" t="n">
         <v>0.57</v>
       </c>
-      <c r="J27" s="32" t="n">
+      <c r="J27" s="33" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="K27" s="32" t="n">
+      <c r="K27" s="33" t="n">
         <v>7.26</v>
       </c>
-      <c r="L27" s="32" t="n">
+      <c r="L27" s="33" t="n">
         <v>7.84</v>
       </c>
-      <c r="M27" s="32" t="n">
+      <c r="M27" s="33" t="n">
         <v>55</v>
       </c>
     </row>
@@ -5281,33 +5224,33 @@
           <t>46 (B-)</t>
         </is>
       </c>
-      <c r="C28" s="32" t="n">
+      <c r="C28" s="33" t="n">
         <v>4.7</v>
       </c>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n">
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="33" t="n">
         <v>1.95</v>
       </c>
-      <c r="F28" s="32" t="n">
+      <c r="F28" s="33" t="n">
         <v>1.92</v>
       </c>
-      <c r="G28" s="32" t="n">
+      <c r="G28" s="33" t="n">
         <v>4.06</v>
       </c>
-      <c r="H28" s="32" t="n"/>
-      <c r="I28" s="32" t="n">
+      <c r="H28" s="33" t="n"/>
+      <c r="I28" s="33" t="n">
         <v>1.27</v>
       </c>
-      <c r="J28" s="32" t="n">
+      <c r="J28" s="33" t="n">
         <v>-22.31</v>
       </c>
-      <c r="K28" s="32" t="n">
+      <c r="K28" s="33" t="n">
         <v>7.12</v>
       </c>
-      <c r="L28" s="32" t="n">
+      <c r="L28" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="M28" s="32" t="n">
+      <c r="M28" s="33" t="n">
         <v>51</v>
       </c>
     </row>
@@ -5322,35 +5265,35 @@
           <t>46 (B-)</t>
         </is>
       </c>
-      <c r="C29" s="32" t="n">
+      <c r="C29" s="33" t="n">
         <v>4.2</v>
       </c>
-      <c r="D29" s="32" t="n">
+      <c r="D29" s="33" t="n">
         <v>-0.04</v>
       </c>
-      <c r="E29" s="32" t="n">
+      <c r="E29" s="33" t="n">
         <v>5.07</v>
       </c>
-      <c r="F29" s="32" t="n">
+      <c r="F29" s="33" t="n">
         <v>1.55</v>
       </c>
-      <c r="G29" s="32" t="n">
+      <c r="G29" s="33" t="n">
         <v>0.36</v>
       </c>
-      <c r="H29" s="32" t="n"/>
-      <c r="I29" s="32" t="n">
+      <c r="H29" s="33" t="n"/>
+      <c r="I29" s="33" t="n">
         <v>0.15</v>
       </c>
-      <c r="J29" s="32" t="n">
+      <c r="J29" s="33" t="n">
         <v>-6.14</v>
       </c>
-      <c r="K29" s="32" t="n">
+      <c r="K29" s="33" t="n">
         <v>7.8</v>
       </c>
-      <c r="L29" s="32" t="n">
+      <c r="L29" s="33" t="n">
         <v>13.33</v>
       </c>
-      <c r="M29" s="32" t="n">
+      <c r="M29" s="33" t="n">
         <v>51</v>
       </c>
     </row>
@@ -5365,35 +5308,35 @@
           <t>45 (B-)</t>
         </is>
       </c>
-      <c r="C30" s="32" t="n">
+      <c r="C30" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="D30" s="32" t="n">
+      <c r="D30" s="33" t="n">
         <v>-2.24</v>
       </c>
-      <c r="E30" s="32" t="n">
+      <c r="E30" s="33" t="n">
         <v>3.57</v>
       </c>
-      <c r="F30" s="32" t="n">
+      <c r="F30" s="33" t="n">
         <v>5.9</v>
       </c>
-      <c r="G30" s="32" t="n">
+      <c r="G30" s="33" t="n">
         <v>2.46</v>
       </c>
-      <c r="H30" s="32" t="n"/>
-      <c r="I30" s="32" t="n">
+      <c r="H30" s="33" t="n"/>
+      <c r="I30" s="33" t="n">
         <v>1.83</v>
       </c>
-      <c r="J30" s="32" t="n">
+      <c r="J30" s="33" t="n">
         <v>-2.43</v>
       </c>
-      <c r="K30" s="32" t="n">
+      <c r="K30" s="33" t="n">
         <v>7.43</v>
       </c>
-      <c r="L30" s="32" t="n">
+      <c r="L30" s="33" t="n">
         <v>6.38</v>
       </c>
-      <c r="M30" s="32" t="n">
+      <c r="M30" s="33" t="n">
         <v>50</v>
       </c>
     </row>
@@ -5408,35 +5351,35 @@
           <t>45 (B-)</t>
         </is>
       </c>
-      <c r="C31" s="32" t="n">
+      <c r="C31" s="33" t="n">
         <v>4.1</v>
       </c>
-      <c r="D31" s="32" t="n">
+      <c r="D31" s="33" t="n">
         <v>-1.7</v>
       </c>
-      <c r="E31" s="32" t="n">
+      <c r="E31" s="33" t="n">
         <v>5.2</v>
       </c>
-      <c r="F31" s="32" t="n">
+      <c r="F31" s="33" t="n">
         <v>1.79</v>
       </c>
-      <c r="G31" s="32" t="n">
+      <c r="G31" s="33" t="n">
         <v>1.98</v>
       </c>
-      <c r="H31" s="32" t="n"/>
-      <c r="I31" s="32" t="n">
+      <c r="H31" s="33" t="n"/>
+      <c r="I31" s="33" t="n">
         <v>-2.44</v>
       </c>
-      <c r="J31" s="32" t="n">
+      <c r="J31" s="33" t="n">
         <v>53.15</v>
       </c>
-      <c r="K31" s="32" t="n">
+      <c r="K31" s="33" t="n">
         <v>7.59</v>
       </c>
-      <c r="L31" s="32" t="n">
+      <c r="L31" s="33" t="n">
         <v>5.88</v>
       </c>
-      <c r="M31" s="32" t="n">
+      <c r="M31" s="33" t="n">
         <v>36</v>
       </c>
     </row>
@@ -5451,35 +5394,35 @@
           <t>45 (B-)</t>
         </is>
       </c>
-      <c r="C32" s="32" t="n">
+      <c r="C32" s="33" t="n">
         <v>3.9</v>
       </c>
-      <c r="D32" s="32" t="n">
+      <c r="D32" s="33" t="n">
         <v>2.87</v>
       </c>
-      <c r="E32" s="32" t="n">
+      <c r="E32" s="33" t="n">
         <v>3.21</v>
       </c>
-      <c r="F32" s="32" t="n">
+      <c r="F32" s="33" t="n">
         <v>4.58</v>
       </c>
-      <c r="G32" s="32" t="n">
+      <c r="G32" s="33" t="n">
         <v>2.78</v>
       </c>
-      <c r="H32" s="32" t="n"/>
-      <c r="I32" s="32" t="n">
+      <c r="H32" s="33" t="n"/>
+      <c r="I32" s="33" t="n">
         <v>0.39</v>
       </c>
-      <c r="J32" s="32" t="n">
+      <c r="J32" s="33" t="n">
         <v>67.45999999999999</v>
       </c>
-      <c r="K32" s="32" t="n">
+      <c r="K32" s="33" t="n">
         <v>8.94</v>
       </c>
-      <c r="L32" s="32" t="n">
+      <c r="L32" s="33" t="n">
         <v>19.35</v>
       </c>
-      <c r="M32" s="32" t="n">
+      <c r="M32" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -5494,35 +5437,35 @@
           <t>43 (C+)</t>
         </is>
       </c>
-      <c r="C33" s="32" t="n">
+      <c r="C33" s="33" t="n">
         <v>3.8</v>
       </c>
-      <c r="D33" s="32" t="n">
+      <c r="D33" s="33" t="n">
         <v>1.66</v>
       </c>
-      <c r="E33" s="32" t="n">
+      <c r="E33" s="33" t="n">
         <v>1.56</v>
       </c>
-      <c r="F33" s="32" t="n">
+      <c r="F33" s="33" t="n">
         <v>4.03</v>
       </c>
-      <c r="G33" s="32" t="n">
+      <c r="G33" s="33" t="n">
         <v>1.76</v>
       </c>
-      <c r="H33" s="32" t="n"/>
-      <c r="I33" s="32" t="n">
+      <c r="H33" s="33" t="n"/>
+      <c r="I33" s="33" t="n">
         <v>-0.36</v>
       </c>
-      <c r="J33" s="32" t="n">
+      <c r="J33" s="33" t="n">
         <v>9.94</v>
       </c>
-      <c r="K33" s="32" t="n">
+      <c r="K33" s="33" t="n">
         <v>7.98</v>
       </c>
-      <c r="L33" s="32" t="n">
+      <c r="L33" s="33" t="n">
         <v>13.79</v>
       </c>
-      <c r="M33" s="32" t="n">
+      <c r="M33" s="33" t="n">
         <v>33</v>
       </c>
     </row>
@@ -5537,35 +5480,35 @@
           <t>41 (C+)</t>
         </is>
       </c>
-      <c r="C34" s="32" t="n">
+      <c r="C34" s="33" t="n">
         <v>5.2</v>
       </c>
-      <c r="D34" s="32" t="n">
+      <c r="D34" s="33" t="n">
         <v>0.88</v>
       </c>
-      <c r="E34" s="32" t="n">
+      <c r="E34" s="33" t="n">
         <v>1.52</v>
       </c>
-      <c r="F34" s="32" t="n">
+      <c r="F34" s="33" t="n">
         <v>2.43</v>
       </c>
-      <c r="G34" s="32" t="n">
+      <c r="G34" s="33" t="n">
         <v>3.28</v>
       </c>
-      <c r="H34" s="32" t="n"/>
-      <c r="I34" s="32" t="n">
+      <c r="H34" s="33" t="n"/>
+      <c r="I34" s="33" t="n">
         <v>1.14</v>
       </c>
-      <c r="J34" s="32" t="n">
+      <c r="J34" s="33" t="n">
         <v>-14.66</v>
       </c>
-      <c r="K34" s="32" t="n">
+      <c r="K34" s="33" t="n">
         <v>7.58</v>
       </c>
-      <c r="L34" s="32" t="n">
+      <c r="L34" s="33" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="M34" s="32" t="n">
+      <c r="M34" s="33" t="n">
         <v>50</v>
       </c>
     </row>
@@ -5580,35 +5523,35 @@
           <t>41 (C+)</t>
         </is>
       </c>
-      <c r="C35" s="32" t="n">
+      <c r="C35" s="33" t="n">
         <v>3.9</v>
       </c>
-      <c r="D35" s="32" t="n">
+      <c r="D35" s="33" t="n">
         <v>-0.14</v>
       </c>
-      <c r="E35" s="32" t="n">
+      <c r="E35" s="33" t="n">
         <v>6.93</v>
       </c>
-      <c r="F35" s="32" t="n">
+      <c r="F35" s="33" t="n">
         <v>3.3</v>
       </c>
-      <c r="G35" s="32" t="n">
+      <c r="G35" s="33" t="n">
         <v>3.22</v>
       </c>
-      <c r="H35" s="32" t="n"/>
-      <c r="I35" s="32" t="n">
+      <c r="H35" s="33" t="n"/>
+      <c r="I35" s="33" t="n">
         <v>0.18</v>
       </c>
-      <c r="J35" s="32" t="n">
+      <c r="J35" s="33" t="n">
         <v>-30.46</v>
       </c>
-      <c r="K35" s="32" t="n">
+      <c r="K35" s="33" t="n">
         <v>6.96</v>
       </c>
-      <c r="L35" s="32" t="n">
+      <c r="L35" s="33" t="n">
         <v>-1.2</v>
       </c>
-      <c r="M35" s="32" t="n">
+      <c r="M35" s="33" t="n">
         <v>82</v>
       </c>
     </row>
@@ -5623,35 +5566,35 @@
           <t>41 (C+)</t>
         </is>
       </c>
-      <c r="C36" s="32" t="n">
+      <c r="C36" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="D36" s="32" t="n">
+      <c r="D36" s="33" t="n">
         <v>-1.05</v>
       </c>
-      <c r="E36" s="32" t="n">
+      <c r="E36" s="33" t="n">
         <v>5.91</v>
       </c>
-      <c r="F36" s="32" t="n">
+      <c r="F36" s="33" t="n">
         <v>2.85</v>
       </c>
-      <c r="G36" s="32" t="n">
+      <c r="G36" s="33" t="n">
         <v>1.44</v>
       </c>
-      <c r="H36" s="32" t="n"/>
-      <c r="I36" s="32" t="n">
+      <c r="H36" s="33" t="n"/>
+      <c r="I36" s="33" t="n">
         <v>-0.55</v>
       </c>
-      <c r="J36" s="32" t="n">
+      <c r="J36" s="33" t="n">
         <v>106.92</v>
       </c>
-      <c r="K36" s="32" t="n">
+      <c r="K36" s="33" t="n">
         <v>6.74</v>
       </c>
-      <c r="L36" s="32" t="n">
+      <c r="L36" s="33" t="n">
         <v>-2.63</v>
       </c>
-      <c r="M36" s="32" t="n">
+      <c r="M36" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -5666,35 +5609,35 @@
           <t>40 (C+)</t>
         </is>
       </c>
-      <c r="C37" s="32" t="n">
+      <c r="C37" s="33" t="n">
         <v>4.9</v>
       </c>
-      <c r="D37" s="32" t="n">
+      <c r="D37" s="33" t="n">
         <v>-2.7</v>
       </c>
-      <c r="E37" s="32" t="n">
+      <c r="E37" s="33" t="n">
         <v>2.39</v>
       </c>
-      <c r="F37" s="32" t="n">
+      <c r="F37" s="33" t="n">
         <v>2.46</v>
       </c>
-      <c r="G37" s="32" t="n">
+      <c r="G37" s="33" t="n">
         <v>3.72</v>
       </c>
-      <c r="H37" s="32" t="n"/>
-      <c r="I37" s="32" t="n">
+      <c r="H37" s="33" t="n"/>
+      <c r="I37" s="33" t="n">
         <v>1.37</v>
       </c>
-      <c r="J37" s="32" t="n">
+      <c r="J37" s="33" t="n">
         <v>-19.67</v>
       </c>
-      <c r="K37" s="32" t="n">
+      <c r="K37" s="33" t="n">
         <v>7.04</v>
       </c>
-      <c r="L37" s="32" t="n">
+      <c r="L37" s="33" t="n">
         <v>-1.54</v>
       </c>
-      <c r="M37" s="32" t="n">
+      <c r="M37" s="33" t="n">
         <v>64</v>
       </c>
     </row>
@@ -5709,35 +5652,35 @@
           <t>38 (C)</t>
         </is>
       </c>
-      <c r="C38" s="32" t="n">
+      <c r="C38" s="33" t="n">
         <v>4.3</v>
       </c>
-      <c r="D38" s="32" t="n">
+      <c r="D38" s="33" t="n">
         <v>1.69</v>
       </c>
-      <c r="E38" s="32" t="n">
+      <c r="E38" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="F38" s="32" t="n">
+      <c r="F38" s="33" t="n">
         <v>7.47</v>
       </c>
-      <c r="G38" s="32" t="n">
+      <c r="G38" s="33" t="n">
         <v>3.1</v>
       </c>
-      <c r="H38" s="32" t="n"/>
-      <c r="I38" s="32" t="n">
+      <c r="H38" s="33" t="n"/>
+      <c r="I38" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="J38" s="32" t="n">
+      <c r="J38" s="33" t="n">
         <v>-8.130000000000001</v>
       </c>
-      <c r="K38" s="32" t="n">
+      <c r="K38" s="33" t="n">
         <v>6.72</v>
       </c>
-      <c r="L38" s="32" t="n">
+      <c r="L38" s="33" t="n">
         <v>3.23</v>
       </c>
-      <c r="M38" s="32" t="n">
+      <c r="M38" s="33" t="n">
         <v>32</v>
       </c>
     </row>
@@ -5752,35 +5695,35 @@
           <t>37 (C)</t>
         </is>
       </c>
-      <c r="C39" s="32" t="n">
+      <c r="C39" s="33" t="n">
         <v>4.4</v>
       </c>
-      <c r="D39" s="32" t="n">
+      <c r="D39" s="33" t="n">
         <v>-0.97</v>
       </c>
-      <c r="E39" s="32" t="n">
+      <c r="E39" s="33" t="n">
         <v>0.01</v>
       </c>
-      <c r="F39" s="32" t="n">
+      <c r="F39" s="33" t="n">
         <v>3.26</v>
       </c>
-      <c r="G39" s="32" t="n">
+      <c r="G39" s="33" t="n">
         <v>1.26</v>
       </c>
-      <c r="H39" s="32" t="n"/>
-      <c r="I39" s="32" t="n">
+      <c r="H39" s="33" t="n"/>
+      <c r="I39" s="33" t="n">
         <v>1.46</v>
       </c>
-      <c r="J39" s="32" t="n">
+      <c r="J39" s="33" t="n">
         <v>9.15</v>
       </c>
-      <c r="K39" s="32" t="n">
+      <c r="K39" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L39" s="32" t="n">
+      <c r="L39" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M39" s="32" t="n">
+      <c r="M39" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -5795,35 +5738,35 @@
           <t>37 (C)</t>
         </is>
       </c>
-      <c r="C40" s="32" t="n">
+      <c r="C40" s="33" t="n">
         <v>7.7</v>
       </c>
-      <c r="D40" s="32" t="n">
+      <c r="D40" s="33" t="n">
         <v>-1.69</v>
       </c>
-      <c r="E40" s="32" t="n">
+      <c r="E40" s="33" t="n">
         <v>5.96</v>
       </c>
-      <c r="F40" s="32" t="n">
+      <c r="F40" s="33" t="n">
         <v>2.61</v>
       </c>
-      <c r="G40" s="32" t="n">
+      <c r="G40" s="33" t="n">
         <v>1.86</v>
       </c>
-      <c r="H40" s="32" t="n"/>
-      <c r="I40" s="32" t="n">
+      <c r="H40" s="33" t="n"/>
+      <c r="I40" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="J40" s="32" t="n">
+      <c r="J40" s="33" t="n">
         <v>-6.89</v>
       </c>
-      <c r="K40" s="32" t="n">
+      <c r="K40" s="33" t="n">
         <v>7.19</v>
       </c>
-      <c r="L40" s="32" t="n">
+      <c r="L40" s="33" t="n">
         <v>5.77</v>
       </c>
-      <c r="M40" s="32" t="n">
+      <c r="M40" s="33" t="n">
         <v>55</v>
       </c>
     </row>
@@ -5838,35 +5781,35 @@
           <t>36 (C)</t>
         </is>
       </c>
-      <c r="C41" s="32" t="n">
+      <c r="C41" s="33" t="n">
         <v>5.3</v>
       </c>
-      <c r="D41" s="32" t="n">
+      <c r="D41" s="33" t="n">
         <v>-1.87</v>
       </c>
-      <c r="E41" s="32" t="n">
+      <c r="E41" s="33" t="n">
         <v>6.17</v>
       </c>
-      <c r="F41" s="32" t="n">
+      <c r="F41" s="33" t="n">
         <v>2.75</v>
       </c>
-      <c r="G41" s="32" t="n">
+      <c r="G41" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="H41" s="32" t="n"/>
-      <c r="I41" s="32" t="n">
+      <c r="H41" s="33" t="n"/>
+      <c r="I41" s="33" t="n">
         <v>0.65</v>
       </c>
-      <c r="J41" s="32" t="n">
+      <c r="J41" s="33" t="n">
         <v>-9.6</v>
       </c>
-      <c r="K41" s="32" t="n">
+      <c r="K41" s="33" t="n">
         <v>7.01</v>
       </c>
-      <c r="L41" s="32" t="n">
+      <c r="L41" s="33" t="n">
         <v>1.72</v>
       </c>
-      <c r="M41" s="32" t="n">
+      <c r="M41" s="33" t="n">
         <v>59</v>
       </c>
     </row>
@@ -5881,35 +5824,35 @@
           <t>36 (C)</t>
         </is>
       </c>
-      <c r="C42" s="32" t="n">
+      <c r="C42" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="D42" s="32" t="n">
+      <c r="D42" s="33" t="n">
         <v>-0.8100000000000001</v>
       </c>
-      <c r="E42" s="32" t="n">
+      <c r="E42" s="33" t="n">
         <v>5.82</v>
       </c>
-      <c r="F42" s="32" t="n">
+      <c r="F42" s="33" t="n">
         <v>2.01</v>
       </c>
-      <c r="G42" s="32" t="n">
+      <c r="G42" s="33" t="n">
         <v>0.68</v>
       </c>
-      <c r="H42" s="32" t="n"/>
-      <c r="I42" s="32" t="n">
+      <c r="H42" s="33" t="n"/>
+      <c r="I42" s="33" t="n">
         <v>-2.07</v>
       </c>
-      <c r="J42" s="32" t="n">
+      <c r="J42" s="33" t="n">
         <v>2.48</v>
       </c>
-      <c r="K42" s="32" t="n">
+      <c r="K42" s="33" t="n">
         <v>7.24</v>
       </c>
-      <c r="L42" s="32" t="n">
+      <c r="L42" s="33" t="n">
         <v>4.08</v>
       </c>
-      <c r="M42" s="32" t="n">
+      <c r="M42" s="33" t="n">
         <v>51</v>
       </c>
     </row>
@@ -5924,35 +5867,35 @@
           <t>36 (C)</t>
         </is>
       </c>
-      <c r="C43" s="32" t="n">
+      <c r="C43" s="33" t="n">
         <v>4.8</v>
       </c>
-      <c r="D43" s="32" t="n">
+      <c r="D43" s="33" t="n">
         <v>0.78</v>
       </c>
-      <c r="E43" s="32" t="n">
+      <c r="E43" s="33" t="n">
         <v>-0.68</v>
       </c>
-      <c r="F43" s="32" t="n">
+      <c r="F43" s="33" t="n">
         <v>2.23</v>
       </c>
-      <c r="G43" s="32" t="n">
+      <c r="G43" s="33" t="n">
         <v>2.86</v>
       </c>
-      <c r="H43" s="32" t="n"/>
-      <c r="I43" s="32" t="n">
+      <c r="H43" s="33" t="n"/>
+      <c r="I43" s="33" t="n">
         <v>0.33</v>
       </c>
-      <c r="J43" s="32" t="n">
+      <c r="J43" s="33" t="n">
         <v>15.03</v>
       </c>
-      <c r="K43" s="32" t="n">
+      <c r="K43" s="33" t="n">
         <v>6.92</v>
       </c>
-      <c r="L43" s="32" t="n">
+      <c r="L43" s="33" t="n">
         <v>-11.94</v>
       </c>
-      <c r="M43" s="32" t="n">
+      <c r="M43" s="33" t="n">
         <v>59</v>
       </c>
     </row>
@@ -5967,35 +5910,35 @@
           <t>35 (C)</t>
         </is>
       </c>
-      <c r="C44" s="32" t="n">
+      <c r="C44" s="33" t="n">
         <v>4.8</v>
       </c>
-      <c r="D44" s="32" t="n">
+      <c r="D44" s="33" t="n">
         <v>0.23</v>
       </c>
-      <c r="E44" s="32" t="n">
+      <c r="E44" s="33" t="n">
         <v>1.33</v>
       </c>
-      <c r="F44" s="32" t="n">
+      <c r="F44" s="33" t="n">
         <v>1.11</v>
       </c>
-      <c r="G44" s="32" t="n">
+      <c r="G44" s="33" t="n">
         <v>2.98</v>
       </c>
-      <c r="H44" s="32" t="n"/>
-      <c r="I44" s="32" t="n">
+      <c r="H44" s="33" t="n"/>
+      <c r="I44" s="33" t="n">
         <v>0.61</v>
       </c>
-      <c r="J44" s="32" t="n">
+      <c r="J44" s="33" t="n">
         <v>5.83</v>
       </c>
-      <c r="K44" s="32" t="n">
+      <c r="K44" s="33" t="n">
         <v>7.01</v>
       </c>
-      <c r="L44" s="32" t="n">
+      <c r="L44" s="33" t="n">
         <v>-1.61</v>
       </c>
-      <c r="M44" s="32" t="n">
+      <c r="M44" s="33" t="n">
         <v>61</v>
       </c>
     </row>
@@ -6010,35 +5953,35 @@
           <t>35 (C)</t>
         </is>
       </c>
-      <c r="C45" s="32" t="n">
+      <c r="C45" s="33" t="n">
         <v>3.4</v>
       </c>
-      <c r="D45" s="32" t="n">
+      <c r="D45" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="E45" s="32" t="n">
+      <c r="E45" s="33" t="n">
         <v>-0.71</v>
       </c>
-      <c r="F45" s="32" t="n">
+      <c r="F45" s="33" t="n">
         <v>5.3</v>
       </c>
-      <c r="G45" s="32" t="n">
+      <c r="G45" s="33" t="n">
         <v>1.44</v>
       </c>
-      <c r="H45" s="32" t="n"/>
-      <c r="I45" s="32" t="n">
+      <c r="H45" s="33" t="n"/>
+      <c r="I45" s="33" t="n">
         <v>-1.33</v>
       </c>
-      <c r="J45" s="32" t="n">
+      <c r="J45" s="33" t="n">
         <v>-0.22</v>
       </c>
-      <c r="K45" s="32" t="n">
+      <c r="K45" s="33" t="n">
         <v>7.98</v>
       </c>
-      <c r="L45" s="32" t="n">
+      <c r="L45" s="33" t="n">
         <v>9.76</v>
       </c>
-      <c r="M45" s="32" t="n">
+      <c r="M45" s="33" t="n">
         <v>45</v>
       </c>
     </row>
@@ -6053,35 +5996,35 @@
           <t>32 (C-)</t>
         </is>
       </c>
-      <c r="C46" s="32" t="n">
+      <c r="C46" s="33" t="n">
         <v>4.8</v>
       </c>
-      <c r="D46" s="32" t="n">
+      <c r="D46" s="33" t="n">
         <v>-1.39</v>
       </c>
-      <c r="E46" s="32" t="n">
+      <c r="E46" s="33" t="n">
         <v>1.15</v>
       </c>
-      <c r="F46" s="32" t="n">
+      <c r="F46" s="33" t="n">
         <v>4.55</v>
       </c>
-      <c r="G46" s="32" t="n">
+      <c r="G46" s="33" t="n">
         <v>0.96</v>
       </c>
-      <c r="H46" s="32" t="n"/>
-      <c r="I46" s="32" t="n">
+      <c r="H46" s="33" t="n"/>
+      <c r="I46" s="33" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="J46" s="32" t="n">
+      <c r="J46" s="33" t="n">
         <v>16.17</v>
       </c>
-      <c r="K46" s="32" t="n">
+      <c r="K46" s="33" t="n">
         <v>6.77</v>
       </c>
-      <c r="L46" s="32" t="n">
+      <c r="L46" s="33" t="n">
         <v>-2.27</v>
       </c>
-      <c r="M46" s="32" t="n">
+      <c r="M46" s="33" t="n">
         <v>43</v>
       </c>
     </row>
@@ -6096,35 +6039,35 @@
           <t>32 (C-)</t>
         </is>
       </c>
-      <c r="C47" s="32" t="n">
+      <c r="C47" s="33" t="n">
         <v>3.8</v>
       </c>
-      <c r="D47" s="32" t="n">
+      <c r="D47" s="33" t="n">
         <v>-0.8</v>
       </c>
-      <c r="E47" s="32" t="n">
+      <c r="E47" s="33" t="n">
         <v>2.59</v>
       </c>
-      <c r="F47" s="32" t="n">
+      <c r="F47" s="33" t="n">
         <v>3.73</v>
       </c>
-      <c r="G47" s="32" t="n">
+      <c r="G47" s="33" t="n">
         <v>1.7</v>
       </c>
-      <c r="H47" s="32" t="n"/>
-      <c r="I47" s="32" t="n">
+      <c r="H47" s="33" t="n"/>
+      <c r="I47" s="33" t="n">
         <v>-0.72</v>
       </c>
-      <c r="J47" s="32" t="n">
+      <c r="J47" s="33" t="n">
         <v>8.220000000000001</v>
       </c>
-      <c r="K47" s="32" t="n">
+      <c r="K47" s="33" t="n">
         <v>5.61</v>
       </c>
-      <c r="L47" s="32" t="n">
+      <c r="L47" s="33" t="n">
         <v>-13.95</v>
       </c>
-      <c r="M47" s="32" t="n">
+      <c r="M47" s="33" t="n">
         <v>37</v>
       </c>
     </row>
@@ -6139,35 +6082,35 @@
           <t>29 (C-)</t>
         </is>
       </c>
-      <c r="C48" s="32" t="n">
+      <c r="C48" s="33" t="n">
         <v>5.4</v>
       </c>
-      <c r="D48" s="32" t="n">
+      <c r="D48" s="33" t="n">
         <v>2.68</v>
       </c>
-      <c r="E48" s="32" t="n">
+      <c r="E48" s="33" t="n">
         <v>1.06</v>
       </c>
-      <c r="F48" s="32" t="n">
+      <c r="F48" s="33" t="n">
         <v>3.24</v>
       </c>
-      <c r="G48" s="32" t="n">
+      <c r="G48" s="33" t="n">
         <v>2.1</v>
       </c>
-      <c r="H48" s="32" t="n"/>
-      <c r="I48" s="32" t="n">
+      <c r="H48" s="33" t="n"/>
+      <c r="I48" s="33" t="n">
         <v>-0.24</v>
       </c>
-      <c r="J48" s="32" t="n">
+      <c r="J48" s="33" t="n">
         <v>-10.99</v>
       </c>
-      <c r="K48" s="32" t="n">
+      <c r="K48" s="33" t="n">
         <v>7.86</v>
       </c>
-      <c r="L48" s="32" t="n">
+      <c r="L48" s="33" t="n">
         <v>8.57</v>
       </c>
-      <c r="M48" s="32" t="n">
+      <c r="M48" s="33" t="n">
         <v>38</v>
       </c>
     </row>
@@ -6182,35 +6125,35 @@
           <t>28 (C-)</t>
         </is>
       </c>
-      <c r="C49" s="32" t="n">
+      <c r="C49" s="33" t="n">
         <v>5.3</v>
       </c>
-      <c r="D49" s="32" t="n">
+      <c r="D49" s="33" t="n">
         <v>-0.53</v>
       </c>
-      <c r="E49" s="32" t="n">
+      <c r="E49" s="33" t="n">
         <v>3.22</v>
       </c>
-      <c r="F49" s="32" t="n">
+      <c r="F49" s="33" t="n">
         <v>3.18</v>
       </c>
-      <c r="G49" s="32" t="n">
+      <c r="G49" s="33" t="n">
         <v>1.92</v>
       </c>
-      <c r="H49" s="32" t="n"/>
-      <c r="I49" s="32" t="n">
+      <c r="H49" s="33" t="n"/>
+      <c r="I49" s="33" t="n">
         <v>0.12</v>
       </c>
-      <c r="J49" s="32" t="n">
+      <c r="J49" s="33" t="n">
         <v>-28.57</v>
       </c>
-      <c r="K49" s="32" t="n">
+      <c r="K49" s="33" t="n">
         <v>6.6</v>
       </c>
-      <c r="L49" s="32" t="n">
+      <c r="L49" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="M49" s="32" t="n">
+      <c r="M49" s="33" t="n">
         <v>33</v>
       </c>
     </row>
@@ -6225,35 +6168,35 @@
           <t>27 (C-)</t>
         </is>
       </c>
-      <c r="C50" s="32" t="n">
+      <c r="C50" s="33" t="n">
         <v>4.2</v>
       </c>
-      <c r="D50" s="32" t="n">
+      <c r="D50" s="33" t="n">
         <v>-8.76</v>
       </c>
-      <c r="E50" s="32" t="n">
+      <c r="E50" s="33" t="n">
         <v>2.03</v>
       </c>
-      <c r="F50" s="32" t="n">
+      <c r="F50" s="33" t="n">
         <v>5.73</v>
       </c>
-      <c r="G50" s="32" t="n">
+      <c r="G50" s="33" t="n">
         <v>0.74</v>
       </c>
-      <c r="H50" s="32" t="n"/>
-      <c r="I50" s="32" t="n">
+      <c r="H50" s="33" t="n"/>
+      <c r="I50" s="33" t="n">
         <v>-0.33</v>
       </c>
-      <c r="J50" s="32" t="n">
+      <c r="J50" s="33" t="n">
         <v>-15.25</v>
       </c>
-      <c r="K50" s="32" t="n">
+      <c r="K50" s="33" t="n">
         <v>5.77</v>
       </c>
-      <c r="L50" s="32" t="n">
+      <c r="L50" s="33" t="n">
         <v>-8.33</v>
       </c>
-      <c r="M50" s="32" t="n">
+      <c r="M50" s="33" t="n">
         <v>33</v>
       </c>
     </row>
@@ -6268,35 +6211,35 @@
           <t>18 (D)</t>
         </is>
       </c>
-      <c r="C51" s="32" t="n">
+      <c r="C51" s="33" t="n">
         <v>5.2</v>
       </c>
-      <c r="D51" s="32" t="n">
+      <c r="D51" s="33" t="n">
         <v>0.08</v>
       </c>
-      <c r="E51" s="32" t="n">
+      <c r="E51" s="33" t="n">
         <v>1.17</v>
       </c>
-      <c r="F51" s="32" t="n">
+      <c r="F51" s="33" t="n">
         <v>3.23</v>
       </c>
-      <c r="G51" s="32" t="n">
+      <c r="G51" s="33" t="n">
         <v>0.44</v>
       </c>
-      <c r="H51" s="32" t="n"/>
-      <c r="I51" s="32" t="n">
+      <c r="H51" s="33" t="n"/>
+      <c r="I51" s="33" t="n">
         <v>-0.47</v>
       </c>
-      <c r="J51" s="32" t="n">
+      <c r="J51" s="33" t="n">
         <v>-27.55</v>
       </c>
-      <c r="K51" s="32" t="n">
+      <c r="K51" s="33" t="n">
         <v>7.53</v>
       </c>
-      <c r="L51" s="32" t="n">
+      <c r="L51" s="33" t="n">
         <v>5.26</v>
       </c>
-      <c r="M51" s="32" t="n">
+      <c r="M51" s="33" t="n">
         <v>40</v>
       </c>
     </row>
@@ -6364,7 +6307,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LFP %</t>
+          <t>CLF YoY %</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">

</xml_diff>